<commit_message>
A2 model doc: 180+ by charge-off-age vintage (< 2 years / 2+ years)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="261">
   <si>
     <t xml:space="preserve">A2 Locatability</t>
   </si>
@@ -811,63 +811,30 @@
     <t xml:space="preserve">Results 180+ by vintage</t>
   </si>
   <si>
-    <t xml:space="preserve">Combined state by vintage at 180+ DPD. Vintage = time since the account first reached 180+ DPD. Yellow = to fill; shares are within each vintage.</t>
+    <t xml:space="preserve">Combined state by vintage at 180+ DPD. Vintage = charge-off age: time since the account was charged off (reached 180+ DPD). Yellow = to fill; shares are within each vintage.</t>
   </si>
   <si>
     <t xml:space="preserve">CC 180+
-&lt; 6 months
+charged off &lt; 2 years
 accounts</t>
   </si>
   <si>
     <t xml:space="preserve">CC 180+
-6–12 months
+charged off 2+ years
 accounts</t>
   </si>
   <si>
-    <t xml:space="preserve">CC 180+
-1–2 years
+    <t xml:space="preserve">RL 180+
+charged off &lt; 2 years
 accounts</t>
   </si>
   <si>
-    <t xml:space="preserve">CC 180+
-2–3 years
+    <t xml:space="preserve">RL 180+
+charged off 2+ years
 accounts</t>
   </si>
   <si>
-    <t xml:space="preserve">CC 180+
-3+ years
-accounts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RL 180+
-&lt; 6 months
-accounts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RL 180+
-6–12 months
-accounts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RL 180+
-1–2 years
-accounts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RL 180+
-2–3 years
-accounts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RL 180+
-3+ years
-accounts</t>
-  </si>
-  <si>
     <t xml:space="preserve">RL vintages cover all three products together; split by product if GRR needs it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vintage bands can be changed in the column headers; the formulas do not depend on them.</t>
   </si>
 </sst>
 </file>
@@ -6331,7 +6298,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:U33"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -6343,18 +6310,6 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6374,8 +6329,6 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -6389,18 +6342,6 @@
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
@@ -6430,42 +6371,6 @@
       <c r="I5" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="J5" s="7" t="s">
-        <v>260</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>261</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>262</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="P5" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="Q5" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="R5" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="S5" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="T5" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="U5" s="7" t="s">
-        <v>207</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
@@ -6491,36 +6396,6 @@
         <f aca="false">IF($H$16=0,"",H6/$H$16)</f>
         <v/>
       </c>
-      <c r="J6" s="43"/>
-      <c r="K6" s="44" t="str">
-        <f aca="false">IF($J$16=0,"",J6/$J$16)</f>
-        <v/>
-      </c>
-      <c r="L6" s="43"/>
-      <c r="M6" s="44" t="str">
-        <f aca="false">IF($L$16=0,"",L6/$L$16)</f>
-        <v/>
-      </c>
-      <c r="N6" s="43"/>
-      <c r="O6" s="44" t="str">
-        <f aca="false">IF($N$16=0,"",N6/$N$16)</f>
-        <v/>
-      </c>
-      <c r="P6" s="43"/>
-      <c r="Q6" s="44" t="str">
-        <f aca="false">IF($P$16=0,"",P6/$P$16)</f>
-        <v/>
-      </c>
-      <c r="R6" s="43"/>
-      <c r="S6" s="44" t="str">
-        <f aca="false">IF($R$16=0,"",R6/$R$16)</f>
-        <v/>
-      </c>
-      <c r="T6" s="43"/>
-      <c r="U6" s="44" t="str">
-        <f aca="false">IF($T$16=0,"",T6/$T$16)</f>
-        <v/>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
@@ -6546,36 +6421,6 @@
         <f aca="false">IF($H$16=0,"",H7/$H$16)</f>
         <v/>
       </c>
-      <c r="J7" s="43"/>
-      <c r="K7" s="44" t="str">
-        <f aca="false">IF($J$16=0,"",J7/$J$16)</f>
-        <v/>
-      </c>
-      <c r="L7" s="43"/>
-      <c r="M7" s="44" t="str">
-        <f aca="false">IF($L$16=0,"",L7/$L$16)</f>
-        <v/>
-      </c>
-      <c r="N7" s="43"/>
-      <c r="O7" s="44" t="str">
-        <f aca="false">IF($N$16=0,"",N7/$N$16)</f>
-        <v/>
-      </c>
-      <c r="P7" s="43"/>
-      <c r="Q7" s="44" t="str">
-        <f aca="false">IF($P$16=0,"",P7/$P$16)</f>
-        <v/>
-      </c>
-      <c r="R7" s="43"/>
-      <c r="S7" s="44" t="str">
-        <f aca="false">IF($R$16=0,"",R7/$R$16)</f>
-        <v/>
-      </c>
-      <c r="T7" s="43"/>
-      <c r="U7" s="44" t="str">
-        <f aca="false">IF($T$16=0,"",T7/$T$16)</f>
-        <v/>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
@@ -6601,36 +6446,6 @@
         <f aca="false">IF($H$16=0,"",H8/$H$16)</f>
         <v/>
       </c>
-      <c r="J8" s="43"/>
-      <c r="K8" s="44" t="str">
-        <f aca="false">IF($J$16=0,"",J8/$J$16)</f>
-        <v/>
-      </c>
-      <c r="L8" s="43"/>
-      <c r="M8" s="44" t="str">
-        <f aca="false">IF($L$16=0,"",L8/$L$16)</f>
-        <v/>
-      </c>
-      <c r="N8" s="43"/>
-      <c r="O8" s="44" t="str">
-        <f aca="false">IF($N$16=0,"",N8/$N$16)</f>
-        <v/>
-      </c>
-      <c r="P8" s="43"/>
-      <c r="Q8" s="44" t="str">
-        <f aca="false">IF($P$16=0,"",P8/$P$16)</f>
-        <v/>
-      </c>
-      <c r="R8" s="43"/>
-      <c r="S8" s="44" t="str">
-        <f aca="false">IF($R$16=0,"",R8/$R$16)</f>
-        <v/>
-      </c>
-      <c r="T8" s="43"/>
-      <c r="U8" s="44" t="str">
-        <f aca="false">IF($T$16=0,"",T8/$T$16)</f>
-        <v/>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
@@ -6656,36 +6471,6 @@
         <f aca="false">IF($H$16=0,"",H9/$H$16)</f>
         <v/>
       </c>
-      <c r="J9" s="43"/>
-      <c r="K9" s="44" t="str">
-        <f aca="false">IF($J$16=0,"",J9/$J$16)</f>
-        <v/>
-      </c>
-      <c r="L9" s="43"/>
-      <c r="M9" s="44" t="str">
-        <f aca="false">IF($L$16=0,"",L9/$L$16)</f>
-        <v/>
-      </c>
-      <c r="N9" s="43"/>
-      <c r="O9" s="44" t="str">
-        <f aca="false">IF($N$16=0,"",N9/$N$16)</f>
-        <v/>
-      </c>
-      <c r="P9" s="43"/>
-      <c r="Q9" s="44" t="str">
-        <f aca="false">IF($P$16=0,"",P9/$P$16)</f>
-        <v/>
-      </c>
-      <c r="R9" s="43"/>
-      <c r="S9" s="44" t="str">
-        <f aca="false">IF($R$16=0,"",R9/$R$16)</f>
-        <v/>
-      </c>
-      <c r="T9" s="43"/>
-      <c r="U9" s="44" t="str">
-        <f aca="false">IF($T$16=0,"",T9/$T$16)</f>
-        <v/>
-      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
@@ -6711,36 +6496,6 @@
         <f aca="false">IF($H$16=0,"",H10/$H$16)</f>
         <v/>
       </c>
-      <c r="J10" s="43"/>
-      <c r="K10" s="44" t="str">
-        <f aca="false">IF($J$16=0,"",J10/$J$16)</f>
-        <v/>
-      </c>
-      <c r="L10" s="43"/>
-      <c r="M10" s="44" t="str">
-        <f aca="false">IF($L$16=0,"",L10/$L$16)</f>
-        <v/>
-      </c>
-      <c r="N10" s="43"/>
-      <c r="O10" s="44" t="str">
-        <f aca="false">IF($N$16=0,"",N10/$N$16)</f>
-        <v/>
-      </c>
-      <c r="P10" s="43"/>
-      <c r="Q10" s="44" t="str">
-        <f aca="false">IF($P$16=0,"",P10/$P$16)</f>
-        <v/>
-      </c>
-      <c r="R10" s="43"/>
-      <c r="S10" s="44" t="str">
-        <f aca="false">IF($R$16=0,"",R10/$R$16)</f>
-        <v/>
-      </c>
-      <c r="T10" s="43"/>
-      <c r="U10" s="44" t="str">
-        <f aca="false">IF($T$16=0,"",T10/$T$16)</f>
-        <v/>
-      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
@@ -6766,36 +6521,6 @@
         <f aca="false">IF($H$16=0,"",H11/$H$16)</f>
         <v/>
       </c>
-      <c r="J11" s="43"/>
-      <c r="K11" s="44" t="str">
-        <f aca="false">IF($J$16=0,"",J11/$J$16)</f>
-        <v/>
-      </c>
-      <c r="L11" s="43"/>
-      <c r="M11" s="44" t="str">
-        <f aca="false">IF($L$16=0,"",L11/$L$16)</f>
-        <v/>
-      </c>
-      <c r="N11" s="43"/>
-      <c r="O11" s="44" t="str">
-        <f aca="false">IF($N$16=0,"",N11/$N$16)</f>
-        <v/>
-      </c>
-      <c r="P11" s="43"/>
-      <c r="Q11" s="44" t="str">
-        <f aca="false">IF($P$16=0,"",P11/$P$16)</f>
-        <v/>
-      </c>
-      <c r="R11" s="43"/>
-      <c r="S11" s="44" t="str">
-        <f aca="false">IF($R$16=0,"",R11/$R$16)</f>
-        <v/>
-      </c>
-      <c r="T11" s="43"/>
-      <c r="U11" s="44" t="str">
-        <f aca="false">IF($T$16=0,"",T11/$T$16)</f>
-        <v/>
-      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
@@ -6821,36 +6546,6 @@
         <f aca="false">IF($H$16=0,"",H12/$H$16)</f>
         <v/>
       </c>
-      <c r="J12" s="43"/>
-      <c r="K12" s="44" t="str">
-        <f aca="false">IF($J$16=0,"",J12/$J$16)</f>
-        <v/>
-      </c>
-      <c r="L12" s="43"/>
-      <c r="M12" s="44" t="str">
-        <f aca="false">IF($L$16=0,"",L12/$L$16)</f>
-        <v/>
-      </c>
-      <c r="N12" s="43"/>
-      <c r="O12" s="44" t="str">
-        <f aca="false">IF($N$16=0,"",N12/$N$16)</f>
-        <v/>
-      </c>
-      <c r="P12" s="43"/>
-      <c r="Q12" s="44" t="str">
-        <f aca="false">IF($P$16=0,"",P12/$P$16)</f>
-        <v/>
-      </c>
-      <c r="R12" s="43"/>
-      <c r="S12" s="44" t="str">
-        <f aca="false">IF($R$16=0,"",R12/$R$16)</f>
-        <v/>
-      </c>
-      <c r="T12" s="43"/>
-      <c r="U12" s="44" t="str">
-        <f aca="false">IF($T$16=0,"",T12/$T$16)</f>
-        <v/>
-      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
@@ -6876,36 +6571,6 @@
         <f aca="false">IF($H$16=0,"",H13/$H$16)</f>
         <v/>
       </c>
-      <c r="J13" s="43"/>
-      <c r="K13" s="44" t="str">
-        <f aca="false">IF($J$16=0,"",J13/$J$16)</f>
-        <v/>
-      </c>
-      <c r="L13" s="43"/>
-      <c r="M13" s="44" t="str">
-        <f aca="false">IF($L$16=0,"",L13/$L$16)</f>
-        <v/>
-      </c>
-      <c r="N13" s="43"/>
-      <c r="O13" s="44" t="str">
-        <f aca="false">IF($N$16=0,"",N13/$N$16)</f>
-        <v/>
-      </c>
-      <c r="P13" s="43"/>
-      <c r="Q13" s="44" t="str">
-        <f aca="false">IF($P$16=0,"",P13/$P$16)</f>
-        <v/>
-      </c>
-      <c r="R13" s="43"/>
-      <c r="S13" s="44" t="str">
-        <f aca="false">IF($R$16=0,"",R13/$R$16)</f>
-        <v/>
-      </c>
-      <c r="T13" s="43"/>
-      <c r="U13" s="44" t="str">
-        <f aca="false">IF($T$16=0,"",T13/$T$16)</f>
-        <v/>
-      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
@@ -6931,36 +6596,6 @@
         <f aca="false">IF($H$16=0,"",H14/$H$16)</f>
         <v/>
       </c>
-      <c r="J14" s="43"/>
-      <c r="K14" s="44" t="str">
-        <f aca="false">IF($J$16=0,"",J14/$J$16)</f>
-        <v/>
-      </c>
-      <c r="L14" s="43"/>
-      <c r="M14" s="44" t="str">
-        <f aca="false">IF($L$16=0,"",L14/$L$16)</f>
-        <v/>
-      </c>
-      <c r="N14" s="43"/>
-      <c r="O14" s="44" t="str">
-        <f aca="false">IF($N$16=0,"",N14/$N$16)</f>
-        <v/>
-      </c>
-      <c r="P14" s="43"/>
-      <c r="Q14" s="44" t="str">
-        <f aca="false">IF($P$16=0,"",P14/$P$16)</f>
-        <v/>
-      </c>
-      <c r="R14" s="43"/>
-      <c r="S14" s="44" t="str">
-        <f aca="false">IF($R$16=0,"",R14/$R$16)</f>
-        <v/>
-      </c>
-      <c r="T14" s="43"/>
-      <c r="U14" s="44" t="str">
-        <f aca="false">IF($T$16=0,"",T14/$T$16)</f>
-        <v/>
-      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
@@ -6986,36 +6621,6 @@
         <f aca="false">IF($H$16=0,"",H15/$H$16)</f>
         <v/>
       </c>
-      <c r="J15" s="43"/>
-      <c r="K15" s="44" t="str">
-        <f aca="false">IF($J$16=0,"",J15/$J$16)</f>
-        <v/>
-      </c>
-      <c r="L15" s="43"/>
-      <c r="M15" s="44" t="str">
-        <f aca="false">IF($L$16=0,"",L15/$L$16)</f>
-        <v/>
-      </c>
-      <c r="N15" s="43"/>
-      <c r="O15" s="44" t="str">
-        <f aca="false">IF($N$16=0,"",N15/$N$16)</f>
-        <v/>
-      </c>
-      <c r="P15" s="43"/>
-      <c r="Q15" s="44" t="str">
-        <f aca="false">IF($P$16=0,"",P15/$P$16)</f>
-        <v/>
-      </c>
-      <c r="R15" s="43"/>
-      <c r="S15" s="44" t="str">
-        <f aca="false">IF($R$16=0,"",R15/$R$16)</f>
-        <v/>
-      </c>
-      <c r="T15" s="43"/>
-      <c r="U15" s="44" t="str">
-        <f aca="false">IF($T$16=0,"",T15/$T$16)</f>
-        <v/>
-      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
@@ -7035,30 +6640,6 @@
       </c>
       <c r="H16" s="46" t="n">
         <f aca="false">SUM(H6:H15)</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="46" t="n">
-        <f aca="false">SUM(J6:J15)</f>
-        <v>0</v>
-      </c>
-      <c r="L16" s="46" t="n">
-        <f aca="false">SUM(L6:L15)</f>
-        <v>0</v>
-      </c>
-      <c r="N16" s="46" t="n">
-        <f aca="false">SUM(N6:N15)</f>
-        <v>0</v>
-      </c>
-      <c r="P16" s="46" t="n">
-        <f aca="false">SUM(P6:P15)</f>
-        <v>0</v>
-      </c>
-      <c r="R16" s="46" t="n">
-        <f aca="false">SUM(R6:R15)</f>
-        <v>0</v>
-      </c>
-      <c r="T16" s="46" t="n">
-        <f aca="false">SUM(T6:T15)</f>
         <v>0</v>
       </c>
     </row>
@@ -7074,18 +6655,6 @@
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
       <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
-      <c r="N18" s="6"/>
-      <c r="O18" s="6"/>
-      <c r="P18" s="6"/>
-      <c r="Q18" s="6"/>
-      <c r="R18" s="6"/>
-      <c r="S18" s="6"/>
-      <c r="T18" s="6"/>
-      <c r="U18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
@@ -7115,42 +6684,6 @@
       <c r="I19" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="J19" s="7" t="s">
-        <v>260</v>
-      </c>
-      <c r="K19" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="L19" s="7" t="s">
-        <v>261</v>
-      </c>
-      <c r="M19" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="N19" s="7" t="s">
-        <v>262</v>
-      </c>
-      <c r="O19" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="P19" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="Q19" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="R19" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="S19" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="T19" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="U19" s="7" t="s">
-        <v>207</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
@@ -7176,36 +6709,6 @@
         <f aca="false">IF($H$23=0,"",H20/$H$23)</f>
         <v/>
       </c>
-      <c r="J20" s="43"/>
-      <c r="K20" s="44" t="str">
-        <f aca="false">IF($J$23=0,"",J20/$J$23)</f>
-        <v/>
-      </c>
-      <c r="L20" s="43"/>
-      <c r="M20" s="44" t="str">
-        <f aca="false">IF($L$23=0,"",L20/$L$23)</f>
-        <v/>
-      </c>
-      <c r="N20" s="43"/>
-      <c r="O20" s="44" t="str">
-        <f aca="false">IF($N$23=0,"",N20/$N$23)</f>
-        <v/>
-      </c>
-      <c r="P20" s="43"/>
-      <c r="Q20" s="44" t="str">
-        <f aca="false">IF($P$23=0,"",P20/$P$23)</f>
-        <v/>
-      </c>
-      <c r="R20" s="43"/>
-      <c r="S20" s="44" t="str">
-        <f aca="false">IF($R$23=0,"",R20/$R$23)</f>
-        <v/>
-      </c>
-      <c r="T20" s="43"/>
-      <c r="U20" s="44" t="str">
-        <f aca="false">IF($T$23=0,"",T20/$T$23)</f>
-        <v/>
-      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
@@ -7231,36 +6734,6 @@
         <f aca="false">IF($H$23=0,"",H21/$H$23)</f>
         <v/>
       </c>
-      <c r="J21" s="43"/>
-      <c r="K21" s="44" t="str">
-        <f aca="false">IF($J$23=0,"",J21/$J$23)</f>
-        <v/>
-      </c>
-      <c r="L21" s="43"/>
-      <c r="M21" s="44" t="str">
-        <f aca="false">IF($L$23=0,"",L21/$L$23)</f>
-        <v/>
-      </c>
-      <c r="N21" s="43"/>
-      <c r="O21" s="44" t="str">
-        <f aca="false">IF($N$23=0,"",N21/$N$23)</f>
-        <v/>
-      </c>
-      <c r="P21" s="43"/>
-      <c r="Q21" s="44" t="str">
-        <f aca="false">IF($P$23=0,"",P21/$P$23)</f>
-        <v/>
-      </c>
-      <c r="R21" s="43"/>
-      <c r="S21" s="44" t="str">
-        <f aca="false">IF($R$23=0,"",R21/$R$23)</f>
-        <v/>
-      </c>
-      <c r="T21" s="43"/>
-      <c r="U21" s="44" t="str">
-        <f aca="false">IF($T$23=0,"",T21/$T$23)</f>
-        <v/>
-      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
@@ -7286,36 +6759,6 @@
         <f aca="false">IF($H$23=0,"",H22/$H$23)</f>
         <v/>
       </c>
-      <c r="J22" s="43"/>
-      <c r="K22" s="44" t="str">
-        <f aca="false">IF($J$23=0,"",J22/$J$23)</f>
-        <v/>
-      </c>
-      <c r="L22" s="43"/>
-      <c r="M22" s="44" t="str">
-        <f aca="false">IF($L$23=0,"",L22/$L$23)</f>
-        <v/>
-      </c>
-      <c r="N22" s="43"/>
-      <c r="O22" s="44" t="str">
-        <f aca="false">IF($N$23=0,"",N22/$N$23)</f>
-        <v/>
-      </c>
-      <c r="P22" s="43"/>
-      <c r="Q22" s="44" t="str">
-        <f aca="false">IF($P$23=0,"",P22/$P$23)</f>
-        <v/>
-      </c>
-      <c r="R22" s="43"/>
-      <c r="S22" s="44" t="str">
-        <f aca="false">IF($R$23=0,"",R22/$R$23)</f>
-        <v/>
-      </c>
-      <c r="T22" s="43"/>
-      <c r="U22" s="44" t="str">
-        <f aca="false">IF($T$23=0,"",T22/$T$23)</f>
-        <v/>
-      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
@@ -7335,30 +6778,6 @@
       </c>
       <c r="H23" s="46" t="n">
         <f aca="false">SUM(H20:H22)</f>
-        <v>0</v>
-      </c>
-      <c r="J23" s="46" t="n">
-        <f aca="false">SUM(J20:J22)</f>
-        <v>0</v>
-      </c>
-      <c r="L23" s="46" t="n">
-        <f aca="false">SUM(L20:L22)</f>
-        <v>0</v>
-      </c>
-      <c r="N23" s="46" t="n">
-        <f aca="false">SUM(N20:N22)</f>
-        <v>0</v>
-      </c>
-      <c r="P23" s="46" t="n">
-        <f aca="false">SUM(P20:P22)</f>
-        <v>0</v>
-      </c>
-      <c r="R23" s="46" t="n">
-        <f aca="false">SUM(R20:R22)</f>
-        <v>0</v>
-      </c>
-      <c r="T23" s="46" t="n">
-        <f aca="false">SUM(T20:T22)</f>
         <v>0</v>
       </c>
     </row>
@@ -7374,18 +6793,6 @@
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
       <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="6"/>
-      <c r="L25" s="6"/>
-      <c r="M25" s="6"/>
-      <c r="N25" s="6"/>
-      <c r="O25" s="6"/>
-      <c r="P25" s="6"/>
-      <c r="Q25" s="6"/>
-      <c r="R25" s="6"/>
-      <c r="S25" s="6"/>
-      <c r="T25" s="6"/>
-      <c r="U25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
@@ -7415,42 +6822,6 @@
       <c r="I26" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="J26" s="7" t="s">
-        <v>260</v>
-      </c>
-      <c r="K26" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="L26" s="7" t="s">
-        <v>261</v>
-      </c>
-      <c r="M26" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="N26" s="7" t="s">
-        <v>262</v>
-      </c>
-      <c r="O26" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="P26" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="Q26" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="R26" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="S26" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="T26" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="U26" s="7" t="s">
-        <v>207</v>
-      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
@@ -7476,36 +6847,6 @@
         <f aca="false">IF($H$30=0,"",H27/$H$30)</f>
         <v/>
       </c>
-      <c r="J27" s="43"/>
-      <c r="K27" s="44" t="str">
-        <f aca="false">IF($J$30=0,"",J27/$J$30)</f>
-        <v/>
-      </c>
-      <c r="L27" s="43"/>
-      <c r="M27" s="44" t="str">
-        <f aca="false">IF($L$30=0,"",L27/$L$30)</f>
-        <v/>
-      </c>
-      <c r="N27" s="43"/>
-      <c r="O27" s="44" t="str">
-        <f aca="false">IF($N$30=0,"",N27/$N$30)</f>
-        <v/>
-      </c>
-      <c r="P27" s="43"/>
-      <c r="Q27" s="44" t="str">
-        <f aca="false">IF($P$30=0,"",P27/$P$30)</f>
-        <v/>
-      </c>
-      <c r="R27" s="43"/>
-      <c r="S27" s="44" t="str">
-        <f aca="false">IF($R$30=0,"",R27/$R$30)</f>
-        <v/>
-      </c>
-      <c r="T27" s="43"/>
-      <c r="U27" s="44" t="str">
-        <f aca="false">IF($T$30=0,"",T27/$T$30)</f>
-        <v/>
-      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
@@ -7531,36 +6872,6 @@
         <f aca="false">IF($H$30=0,"",H28/$H$30)</f>
         <v/>
       </c>
-      <c r="J28" s="43"/>
-      <c r="K28" s="44" t="str">
-        <f aca="false">IF($J$30=0,"",J28/$J$30)</f>
-        <v/>
-      </c>
-      <c r="L28" s="43"/>
-      <c r="M28" s="44" t="str">
-        <f aca="false">IF($L$30=0,"",L28/$L$30)</f>
-        <v/>
-      </c>
-      <c r="N28" s="43"/>
-      <c r="O28" s="44" t="str">
-        <f aca="false">IF($N$30=0,"",N28/$N$30)</f>
-        <v/>
-      </c>
-      <c r="P28" s="43"/>
-      <c r="Q28" s="44" t="str">
-        <f aca="false">IF($P$30=0,"",P28/$P$30)</f>
-        <v/>
-      </c>
-      <c r="R28" s="43"/>
-      <c r="S28" s="44" t="str">
-        <f aca="false">IF($R$30=0,"",R28/$R$30)</f>
-        <v/>
-      </c>
-      <c r="T28" s="43"/>
-      <c r="U28" s="44" t="str">
-        <f aca="false">IF($T$30=0,"",T28/$T$30)</f>
-        <v/>
-      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
@@ -7586,36 +6897,6 @@
         <f aca="false">IF($H$30=0,"",H29/$H$30)</f>
         <v/>
       </c>
-      <c r="J29" s="43"/>
-      <c r="K29" s="44" t="str">
-        <f aca="false">IF($J$30=0,"",J29/$J$30)</f>
-        <v/>
-      </c>
-      <c r="L29" s="43"/>
-      <c r="M29" s="44" t="str">
-        <f aca="false">IF($L$30=0,"",L29/$L$30)</f>
-        <v/>
-      </c>
-      <c r="N29" s="43"/>
-      <c r="O29" s="44" t="str">
-        <f aca="false">IF($N$30=0,"",N29/$N$30)</f>
-        <v/>
-      </c>
-      <c r="P29" s="43"/>
-      <c r="Q29" s="44" t="str">
-        <f aca="false">IF($P$30=0,"",P29/$P$30)</f>
-        <v/>
-      </c>
-      <c r="R29" s="43"/>
-      <c r="S29" s="44" t="str">
-        <f aca="false">IF($R$30=0,"",R29/$R$30)</f>
-        <v/>
-      </c>
-      <c r="T29" s="43"/>
-      <c r="U29" s="44" t="str">
-        <f aca="false">IF($T$30=0,"",T29/$T$30)</f>
-        <v/>
-      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="22" t="s">
@@ -7637,34 +6918,10 @@
         <f aca="false">SUM(H27:H29)</f>
         <v>0</v>
       </c>
-      <c r="J30" s="46" t="n">
-        <f aca="false">SUM(J27:J29)</f>
-        <v>0</v>
-      </c>
-      <c r="L30" s="46" t="n">
-        <f aca="false">SUM(L27:L29)</f>
-        <v>0</v>
-      </c>
-      <c r="N30" s="46" t="n">
-        <f aca="false">SUM(N27:N29)</f>
-        <v>0</v>
-      </c>
-      <c r="P30" s="46" t="n">
-        <f aca="false">SUM(P27:P29)</f>
-        <v>0</v>
-      </c>
-      <c r="R30" s="46" t="n">
-        <f aca="false">SUM(R27:R29)</f>
-        <v>0</v>
-      </c>
-      <c r="T30" s="46" t="n">
-        <f aca="false">SUM(T27:T29)</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -7674,29 +6931,11 @@
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A32:K32"/>
-    <mergeCell ref="A33:K33"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A32:I32"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
A2 model doc: vintages named early-stage / late-stage charge-off
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -811,26 +811,30 @@
     <t xml:space="preserve">Results 180+ by vintage</t>
   </si>
   <si>
-    <t xml:space="preserve">Combined state by vintage at 180+ DPD. Vintage = charge-off age: time since the account was charged off (reached 180+ DPD). Yellow = to fill; shares are within each vintage.</t>
+    <t xml:space="preserve">Combined state by vintage at 180+ DPD. Vintage = charge-off age: early-stage = charged off less than 2 years ago, late-stage = 2 years or more (charge-off = reaching 180+ DPD). Yellow = to fill; shares are within each vintage.</t>
   </si>
   <si>
     <t xml:space="preserve">CC 180+
-charged off &lt; 2 years
+early-stage charge-off
+(&lt; 2 years)
 accounts</t>
   </si>
   <si>
     <t xml:space="preserve">CC 180+
-charged off 2+ years
+late-stage charge-off
+(2+ years)
 accounts</t>
   </si>
   <si>
     <t xml:space="preserve">RL 180+
-charged off &lt; 2 years
+early-stage charge-off
+(&lt; 2 years)
 accounts</t>
   </si>
   <si>
     <t xml:space="preserve">RL 180+
-charged off 2+ years
+late-stage charge-off
+(2+ years)
 accounts</t>
   </si>
   <si>

</xml_diff>

<commit_message>
A2: only in-person card use (shop, ATM) is location evidence; online and transfers excluded (D-A2-13)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="264">
   <si>
     <t xml:space="preserve">A2 Locatability</t>
   </si>
@@ -43,7 +43,7 @@
     <t xml:space="preserve">Location</t>
   </si>
   <si>
-    <t xml:space="preserve">Where the customer is, from what they do: digital-banking logins, card and current/savings (CASA) spending on all the customer's accounts, travel purchases, and a collector's note that the customer left the country.</t>
+    <t xml:space="preserve">Where the customer is, from what they do: digital-banking logins, in-person card use (shop payments, ATM withdrawals) on all the customer's cards and accounts, travel purchases, and a collector's note that the customer left the country.</t>
   </si>
   <si>
     <t xml:space="preserve">Reachability</t>
@@ -220,10 +220,10 @@
     <t xml:space="preserve">Any of, at any age up to the scoring date: a collector's deceased result (DECEASED, DECEASED CLAIMED, DECEASED OR EXPIRED, …); card block code D on the latest contract snapshot (cards only); the deceased flag on the customer's latest demographics record.</t>
   </si>
   <si>
-    <t xml:space="preserve">The latest foreign evidence is later than the latest UAE evidence, or there is no UAE evidence. Foreign evidence = a login from abroad, card or CASA spending abroad, a collector's departure note (any age), or a travel purchase in the last 12 months.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The latest evidence is a UAE login or UAE spending (not a travel purchase), dated within the window. Same day as foreign evidence: the UAE evidence wins.</t>
+    <t xml:space="preserve">The latest foreign evidence is later than the latest UAE evidence, or there is no UAE evidence. Foreign evidence = a login from abroad, a shop payment or ATM withdrawal abroad, a collector's departure note (any age), or a travel purchase in the last 12 months.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The latest evidence is a UAE login or a shop payment or ATM withdrawal in the UAE (not a travel purchase), dated within the window. Same day as foreign evidence: the UAE evidence wins.</t>
   </si>
   <si>
     <t xml:space="preserve">No evidence at all, or the latest evidence is in the UAE but older than the window.</t>
@@ -289,10 +289,10 @@
     <t xml:space="preserve">Codes</t>
   </si>
   <si>
-    <t xml:space="preserve">U: UAE login / spend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F: abroad login / spend</t>
+    <t xml:space="preserve">U: UAE login / card use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F: abroad login / card use</t>
   </si>
   <si>
     <t xml:space="preserve">T: travel purchase</t>
@@ -346,7 +346,7 @@
     <t xml:space="preserve">U</t>
   </si>
   <si>
-    <t xml:space="preserve">Spent abroad 8 months ago, UAE spending last month.</t>
+    <t xml:space="preserve">Used the card abroad 8 months ago, in the UAE last month.</t>
   </si>
   <si>
     <t xml:space="preserve">T</t>
@@ -379,7 +379,7 @@
     <t xml:space="preserve">Only a travel purchase older than 12 months: no evidence. (T at -15 not shown)</t>
   </si>
   <si>
-    <t xml:space="preserve">No logins and no card or CASA activity on record.</t>
+    <t xml:space="preserve">No logins and no in-person card use on record.</t>
   </si>
   <si>
     <t xml:space="preserve">Reachability — one code per call day, oldest first within a month</t>
@@ -487,10 +487,10 @@
     <t xml:space="preserve">Digital-banking login history</t>
   </si>
   <si>
-    <t xml:space="preserve">Card spending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UAE or foreign, by merchant country</t>
+    <t xml:space="preserve">Credit card used in person (shop, ATM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UAE or foreign, by where it was used</t>
   </si>
   <si>
     <t xml:space="preserve">Customer (all cards)</t>
@@ -499,16 +499,25 @@
     <t xml:space="preserve">Card transactions</t>
   </si>
   <si>
-    <t xml:space="preserve">CASA spending (debit card, ATM, transfers)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UAE or foreign</t>
+    <t xml:space="preserve">Debit card used in person (shop, ATM)</t>
   </si>
   <si>
     <t xml:space="preserve">Customer (all CASA accounts)</t>
   </si>
   <si>
     <t xml:space="preserve">CASA transactions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Online purchases, transfers and remittances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paying a foreign shop online or sending money home does not show where the customer is</t>
   </si>
   <si>
     <t xml:space="preserve">Travel purchase (airline, cruise, travel agency)</t>
@@ -742,10 +751,10 @@
     <t xml:space="preserve">Login from abroad</t>
   </si>
   <si>
-    <t xml:space="preserve">Card spending abroad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CASA spending abroad</t>
+    <t xml:space="preserve">Credit card used abroad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debit card / ATM used abroad</t>
   </si>
   <si>
     <t xml:space="preserve">Travel purchase</t>
@@ -760,10 +769,10 @@
     <t xml:space="preserve">UAE login</t>
   </si>
   <si>
-    <t xml:space="preserve">UAE card spending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UAE CASA spending</t>
+    <t xml:space="preserve">Credit card used in the UAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debit card / ATM used in the UAE</t>
   </si>
   <si>
     <t xml:space="preserve">Why Location is Unknown</t>
@@ -3042,7 +3051,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -3135,121 +3144,121 @@
         <v>4</v>
       </c>
       <c r="C7" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>158</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>159</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>151</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>161</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>4</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>162</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>163</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="F9" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="B10" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="9" t="s">
+      <c r="E10" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="D10" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>71</v>
-      </c>
       <c r="F10" s="9" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>71</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>10</v>
+        <v>176</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>168</v>
+        <v>71</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>10</v>
@@ -3258,18 +3267,18 @@
         <v>10</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>10</v>
@@ -3278,13 +3287,33 @@
         <v>10</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>180</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>181</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -3317,12 +3346,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3330,13 +3359,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>103</v>
@@ -3347,13 +3376,13 @@
         <v>71</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3361,13 +3390,13 @@
         <v>71</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C6" s="42" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3375,13 +3404,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C7" s="42" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3389,13 +3418,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C8" s="42" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3403,13 +3432,13 @@
         <v>6</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C9" s="42" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3417,13 +3446,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C10" s="42" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -3473,12 +3502,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3493,7 +3522,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -3521,64 +3550,64 @@
         <v>15</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="Q5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="T5" s="7" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="U5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3644,7 +3673,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B7" s="43"/>
       <c r="C7" s="44" t="str">
@@ -3705,7 +3734,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B8" s="43"/>
       <c r="C8" s="44" t="str">
@@ -3766,7 +3795,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B9" s="43"/>
       <c r="C9" s="44" t="str">
@@ -3827,7 +3856,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B10" s="43"/>
       <c r="C10" s="44" t="str">
@@ -3888,7 +3917,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B11" s="43"/>
       <c r="C11" s="44" t="str">
@@ -3949,7 +3978,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B12" s="43"/>
       <c r="C12" s="44" t="str">
@@ -4010,7 +4039,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B13" s="43"/>
       <c r="C13" s="44" t="str">
@@ -4071,7 +4100,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B14" s="43"/>
       <c r="C14" s="44" t="str">
@@ -4132,7 +4161,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B15" s="43"/>
       <c r="C15" s="44" t="str">
@@ -4193,7 +4222,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B16" s="46" t="n">
         <f aca="false">SUM(B6:B15)</f>
@@ -4238,7 +4267,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -4266,64 +4295,64 @@
         <v>15</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="N19" s="7" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="P19" s="7" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="Q19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R19" s="7" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="S19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="T19" s="7" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="U19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4511,7 +4540,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B23" s="46" t="n">
         <f aca="false">SUM(B20:B22)</f>
@@ -4556,7 +4585,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -4584,64 +4613,64 @@
         <v>15</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="N26" s="7" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="O26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="P26" s="7" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="Q26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R26" s="7" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="S26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="T26" s="7" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="U26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4829,7 +4858,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="22" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B30" s="46" t="n">
         <f aca="false">SUM(B27:B29)</f>
@@ -4874,7 +4903,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -4899,72 +4928,72 @@
     </row>
     <row r="33" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="M33" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="N33" s="7" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="O33" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="P33" s="7" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="Q33" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R33" s="7" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="S33" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="T33" s="7" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="U33" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B34" s="43"/>
       <c r="C34" s="44" t="str">
@@ -5025,7 +5054,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B35" s="43"/>
       <c r="C35" s="44" t="str">
@@ -5086,7 +5115,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B36" s="43"/>
       <c r="C36" s="44" t="str">
@@ -5147,7 +5176,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="17" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B37" s="43"/>
       <c r="C37" s="44" t="str">
@@ -5208,7 +5237,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="17" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B38" s="43"/>
       <c r="C38" s="44" t="str">
@@ -5314,7 +5343,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
@@ -5339,72 +5368,72 @@
     </row>
     <row r="42" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H42" s="7" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="I42" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="J42" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="K42" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="L42" s="7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="M42" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="N42" s="7" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="O42" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="P42" s="7" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="Q42" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R42" s="7" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="S42" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="T42" s="7" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="U42" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="17" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B43" s="43"/>
       <c r="C43" s="44" t="str">
@@ -5465,7 +5494,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="17" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B44" s="43"/>
       <c r="C44" s="44" t="str">
@@ -5526,7 +5555,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="17" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B45" s="43"/>
       <c r="C45" s="44" t="str">
@@ -5632,7 +5661,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
@@ -5657,72 +5686,72 @@
     </row>
     <row r="49" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="I49" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="J49" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="K49" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="L49" s="7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="M49" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="N49" s="7" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="O49" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="P49" s="7" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="Q49" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R49" s="7" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="S49" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="T49" s="7" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="U49" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="17" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B50" s="43"/>
       <c r="C50" s="44" t="str">
@@ -5783,7 +5812,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="17" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B51" s="43"/>
       <c r="C51" s="44" t="str">
@@ -5844,7 +5873,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="22" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B52" s="46" t="n">
         <f aca="false">SUM(B50:B51)</f>
@@ -5889,7 +5918,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
@@ -5914,72 +5943,72 @@
     </row>
     <row r="55" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="I55" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="J55" s="7" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="K55" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="L55" s="7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="M55" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="N55" s="7" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="O55" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="P55" s="7" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="Q55" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R55" s="7" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="S55" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="T55" s="7" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="U55" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="17" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B56" s="43"/>
       <c r="C56" s="44" t="str">
@@ -6040,7 +6069,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="17" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B57" s="43"/>
       <c r="C57" s="44" t="str">
@@ -6101,7 +6130,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="22" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B58" s="46" t="n">
         <f aca="false">SUM(B56:B57)</f>
@@ -6146,7 +6175,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -6171,7 +6200,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="47" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B61" s="43"/>
       <c r="D61" s="43"/>
@@ -6192,7 +6221,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="22" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B62" s="49" t="str">
         <f aca="false">IF(B61=0,"",B16/B61)</f>
@@ -6237,7 +6266,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -6252,7 +6281,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -6267,7 +6296,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -6318,12 +6347,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6336,7 +6365,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -6352,28 +6381,28 @@
         <v>15</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6403,7 +6432,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B7" s="43"/>
       <c r="C7" s="44" t="str">
@@ -6428,7 +6457,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B8" s="43"/>
       <c r="C8" s="44" t="str">
@@ -6453,7 +6482,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B9" s="43"/>
       <c r="C9" s="44" t="str">
@@ -6478,7 +6507,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B10" s="43"/>
       <c r="C10" s="44" t="str">
@@ -6503,7 +6532,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B11" s="43"/>
       <c r="C11" s="44" t="str">
@@ -6528,7 +6557,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B12" s="43"/>
       <c r="C12" s="44" t="str">
@@ -6553,7 +6582,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B13" s="43"/>
       <c r="C13" s="44" t="str">
@@ -6578,7 +6607,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B14" s="43"/>
       <c r="C14" s="44" t="str">
@@ -6603,7 +6632,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B15" s="43"/>
       <c r="C15" s="44" t="str">
@@ -6628,7 +6657,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B16" s="46" t="n">
         <f aca="false">SUM(B6:B15)</f>
@@ -6665,28 +6694,28 @@
         <v>15</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6766,7 +6795,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B23" s="46" t="n">
         <f aca="false">SUM(B20:B22)</f>
@@ -6803,28 +6832,28 @@
         <v>15</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6904,7 +6933,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="22" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B30" s="46" t="n">
         <f aca="false">SUM(B27:B29)</f>
@@ -6925,7 +6954,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>

</xml_diff>

<commit_message>
A2: Skip rule worded unambiguously (needs foreign evidence; no evidence is Unknown)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="162">
   <si>
     <t xml:space="preserve">A2 Locatability</t>
   </si>
@@ -200,25 +200,28 @@
     <t xml:space="preserve">Rule 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Latest foreign evidence is later than the latest UAE evidence, or there is no UAE evidence.</t>
+    <t xml:space="preserve">There is foreign evidence, and it is later than any UAE evidence.</t>
   </si>
   <si>
     <t xml:space="preserve">Rule 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Latest UAE evidence is within the window (on the same day as foreign evidence, UAE wins).</t>
+    <t xml:space="preserve">The latest evidence is UAE evidence within the window (on the same day as foreign evidence, UAE wins).</t>
   </si>
   <si>
     <t xml:space="preserve">Rule 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Otherwise: no evidence at all, or the latest UAE evidence is older than the window.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last 3 call days all failed, the oldest within the window, and no contact since.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last contact is within the window.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Otherwise.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last 3 call days all failed, the oldest within the window, and no contact since.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last contact is within the window.</t>
   </si>
   <si>
     <t xml:space="preserve">Deceased flag is set, at any date. Overrides both dimensions.</t>
@@ -1635,7 +1638,7 @@
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
     </row>
-    <row r="14" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
         <v>57</v>
       </c>
@@ -1659,7 +1662,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
         <v>61</v>
       </c>
@@ -1708,7 +1711,7 @@
         <v>61</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C21" s="21"/>
       <c r="D21" s="12" t="s">
@@ -1728,7 +1731,7 @@
         <v>57</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C24" s="21"/>
       <c r="D24" s="13" t="s">
@@ -1737,7 +1740,7 @@
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1745,74 +1748,74 @@
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C28" s="18"/>
       <c r="D28" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C29" s="18"/>
       <c r="D29" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C30" s="18"/>
       <c r="D30" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C31" s="18"/>
       <c r="D31" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C32" s="18"/>
       <c r="D32" s="19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1864,12 +1867,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1899,22 +1902,22 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C5" s="23"/>
       <c r="D5" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E5" s="24"/>
       <c r="F5" s="24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G5" s="24"/>
       <c r="H5" s="24" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I5" s="24"/>
     </row>
@@ -1923,34 +1926,34 @@
         <v>11</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H6" s="25" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I6" s="25" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J6" s="25" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1960,18 +1963,18 @@
       <c r="B7" s="26"/>
       <c r="C7" s="26"/>
       <c r="D7" s="15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E7" s="26"/>
       <c r="F7" s="26"/>
       <c r="G7" s="26"/>
       <c r="H7" s="27"/>
       <c r="I7" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J7" s="27"/>
       <c r="K7" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1983,16 +1986,16 @@
       <c r="D8" s="26"/>
       <c r="E8" s="26"/>
       <c r="F8" s="15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G8" s="26"/>
       <c r="H8" s="27"/>
       <c r="I8" s="27"/>
       <c r="J8" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2005,15 +2008,15 @@
       <c r="E9" s="26"/>
       <c r="F9" s="26"/>
       <c r="G9" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H9" s="27"/>
       <c r="I9" s="15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J9" s="27"/>
       <c r="K9" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2021,7 +2024,7 @@
         <v>16</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
@@ -2032,7 +2035,7 @@
       <c r="I10" s="27"/>
       <c r="J10" s="27"/>
       <c r="K10" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2041,19 +2044,19 @@
       </c>
       <c r="B11" s="26"/>
       <c r="C11" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D11" s="26"/>
       <c r="E11" s="26"/>
       <c r="F11" s="15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G11" s="26"/>
       <c r="H11" s="27"/>
       <c r="I11" s="27"/>
       <c r="J11" s="27"/>
       <c r="K11" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2064,7 +2067,7 @@
       <c r="C12" s="26"/>
       <c r="D12" s="26"/>
       <c r="E12" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F12" s="26"/>
       <c r="G12" s="26"/>
@@ -2072,7 +2075,7 @@
       <c r="I12" s="27"/>
       <c r="J12" s="27"/>
       <c r="K12" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2089,7 +2092,7 @@
       <c r="I13" s="27"/>
       <c r="J13" s="27"/>
       <c r="K13" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2109,22 +2112,22 @@
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C16" s="23"/>
       <c r="D16" s="23" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E16" s="23"/>
       <c r="F16" s="24" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G16" s="24"/>
       <c r="H16" s="24" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I16" s="24"/>
     </row>
@@ -2133,34 +2136,34 @@
         <v>11</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H17" s="25" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I17" s="25" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J17" s="25" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2175,11 +2178,11 @@
       <c r="G18" s="26"/>
       <c r="H18" s="27"/>
       <c r="I18" s="14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J18" s="27"/>
       <c r="K18" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2193,12 +2196,12 @@
       <c r="F19" s="26"/>
       <c r="G19" s="26"/>
       <c r="H19" s="14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I19" s="27"/>
       <c r="J19" s="27"/>
       <c r="K19" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2212,16 +2215,16 @@
       <c r="F20" s="26"/>
       <c r="G20" s="26"/>
       <c r="H20" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J20" s="14" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2235,16 +2238,16 @@
       <c r="F21" s="26"/>
       <c r="G21" s="26"/>
       <c r="H21" s="14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J21" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2256,18 +2259,18 @@
       <c r="D22" s="26"/>
       <c r="E22" s="26"/>
       <c r="F22" s="14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G22" s="26"/>
       <c r="H22" s="27"/>
       <c r="I22" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J22" s="15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K22" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2277,20 +2280,20 @@
       <c r="B23" s="26"/>
       <c r="C23" s="26"/>
       <c r="D23" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G23" s="26"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
       <c r="J23" s="27"/>
       <c r="K23" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2307,12 +2310,12 @@
       <c r="I24" s="27"/>
       <c r="J24" s="27"/>
       <c r="K24" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -2381,12 +2384,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2412,7 +2415,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -2444,64 +2447,64 @@
         <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E6" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>134</v>
-      </c>
       <c r="G6" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="V6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3144,7 +3147,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="31" t="n">
@@ -3200,7 +3203,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B18" s="18"/>
       <c r="C18" s="28"/>
@@ -3232,7 +3235,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="32" t="str">
@@ -3318,64 +3321,64 @@
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E22" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>134</v>
-      </c>
       <c r="G22" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="N22" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O22" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q22" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R22" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S22" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T22" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="U22" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="V22" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3566,7 +3569,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="31" t="n">
@@ -3652,64 +3655,64 @@
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E29" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F29" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>134</v>
-      </c>
       <c r="G29" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="N29" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O29" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P29" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q29" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R29" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S29" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T29" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="U29" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="V29" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3900,7 +3903,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="31" t="n">
@@ -3956,7 +3959,7 @@
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -3982,73 +3985,73 @@
     </row>
     <row r="36" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E36" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F36" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="F36" s="7" t="s">
-        <v>134</v>
-      </c>
       <c r="G36" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M36" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="N36" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O36" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P36" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q36" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R36" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S36" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T36" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="U36" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="V36" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B37" s="12"/>
       <c r="C37" s="28"/>
@@ -4110,7 +4113,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="28"/>
@@ -4172,7 +4175,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B39" s="12"/>
       <c r="C39" s="28"/>
@@ -4234,7 +4237,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B40" s="12"/>
       <c r="C40" s="28"/>
@@ -4296,7 +4299,7 @@
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -4322,7 +4325,7 @@
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -4402,12 +4405,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4421,7 +4424,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -4441,28 +4444,28 @@
         <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4745,7 +4748,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="31" t="n">

</xml_diff>

<commit_message>
A2: same-day UAE and foreign evidence -> foreign wins (D-A2-14); login fix needs no timestamps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -200,13 +200,13 @@
     <t xml:space="preserve">Rule 1</t>
   </si>
   <si>
-    <t xml:space="preserve">There is foreign evidence, and it is later than any UAE evidence.</t>
+    <t xml:space="preserve">There is foreign evidence, and it is on or after the date of the latest UAE evidence (on the same day, foreign wins).</t>
   </si>
   <si>
     <t xml:space="preserve">Rule 2</t>
   </si>
   <si>
-    <t xml:space="preserve">The latest evidence is UAE evidence within the window (on the same day as foreign evidence, UAE wins).</t>
+    <t xml:space="preserve">The latest evidence is UAE evidence within the window.</t>
   </si>
   <si>
     <t xml:space="preserve">Rule 3</t>
@@ -1638,7 +1638,7 @@
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
     </row>
-    <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
         <v>57</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
         <v>59</v>
       </c>

</xml_diff>

<commit_message>
A2 model doc: location evidence table makes the 12-month travel rule explicit; travel examples (back, too old)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="186">
   <si>
     <t xml:space="preserve">A2 Locatability</t>
   </si>
@@ -155,6 +155,63 @@
     <t xml:space="preserve">What the model computes for each account at the scoring date, and the rules that turn it into states. Within a dimension, the first rule that holds decides.</t>
   </si>
   <si>
+    <t xml:space="preserve">Location evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What counts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UAE or foreign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Counts for</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Digital-banking login.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">By login country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Card use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In-person card use (shop payment, ATM withdrawal) on any of the customer's cards and accounts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">By where it was used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel purchase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airline, cruise or travel-agency purchase, dated on the purchase day.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foreign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 months; older ones are ignored</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collector note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer left the country (final exit visa included).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A travel purchase is foreign evidence like any other: it gives Skip unless UAE evidence comes after it (the customer came back or never left).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Features</t>
   </si>
   <si>
@@ -167,13 +224,13 @@
     <t xml:space="preserve">Latest UAE evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Date of the most recent login from the UAE, or in-person card use in the UAE (shop payment, ATM withdrawal) on any of the customer's cards and accounts.</t>
+    <t xml:space="preserve">Most recent date of UAE evidence.</t>
   </si>
   <si>
     <t xml:space="preserve">Latest foreign evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Date of the most recent login from abroad, in-person card use abroad, travel purchase (airline, cruise, travel agency) in the last 12 months, or collector note that the customer left the country.</t>
+    <t xml:space="preserve">Most recent date of foreign evidence, travel purchases included while under 12 months old.</t>
   </si>
   <si>
     <t xml:space="preserve">Last contact</t>
@@ -257,9 +314,6 @@
     <t xml:space="preserve">No sign of return means still abroad.</t>
   </si>
   <si>
-    <t xml:space="preserve">Travel purchase</t>
-  </si>
-  <si>
     <t xml:space="preserve">Counts for 12 months.</t>
   </si>
   <si>
@@ -305,6 +359,18 @@
     <t xml:space="preserve">X  left UAE</t>
   </si>
   <si>
+    <t xml:space="preserve">-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-9</t>
+  </si>
+  <si>
     <t xml:space="preserve">-8</t>
   </si>
   <si>
@@ -341,6 +407,12 @@
     <t xml:space="preserve">Abroad 6 months ago; card used in the UAE last month.</t>
   </si>
   <si>
+    <t xml:space="preserve">T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flight bought, then card used in the UAE.</t>
+  </si>
+  <si>
     <t xml:space="preserve">X</t>
   </si>
   <si>
@@ -353,10 +425,10 @@
     <t xml:space="preserve">Last seen abroad 8 months ago, nothing since.</t>
   </si>
   <si>
-    <t xml:space="preserve">T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bought a flight 4 months ago, no UAE activity since.</t>
+    <t xml:space="preserve">Flight bought 4 months ago, no UAE activity since.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only a flight bought 12 months ago: too old, ignored.</t>
   </si>
   <si>
     <t xml:space="preserve">Last UAE activity is older than the window.</t>
@@ -1520,7 +1592,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -1557,290 +1629,377 @@
       <c r="B5" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="7"/>
+      <c r="C5" s="7" t="s">
+        <v>46</v>
+      </c>
       <c r="D5" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="19" t="s">
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="18"/>
+      <c r="D14" s="19" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="19" t="s">
+    <row r="15" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="18"/>
+      <c r="D15" s="19" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="19" t="s">
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" s="18"/>
+      <c r="D16" s="19" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="19" t="s">
+    <row r="17" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="18"/>
+      <c r="D17" s="19" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="19" t="s">
+    <row r="18" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" s="18"/>
+      <c r="D18" s="19" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-    </row>
-    <row r="14" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="21"/>
-      <c r="D14" s="11" t="s">
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="C22" s="21"/>
+      <c r="D22" s="11" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="21"/>
-      <c r="D15" s="8" t="s">
+    <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" s="21"/>
+      <c r="D23" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="B16" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" s="21"/>
-      <c r="D16" s="12" t="s">
+    <row r="24" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24" s="21"/>
+      <c r="D24" s="12" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="B19" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="C19" s="21"/>
-      <c r="D19" s="11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="C20" s="21"/>
-      <c r="D20" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="B21" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C21" s="21"/>
-      <c r="D21" s="12" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="13" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>67</v>
+        <v>6</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
     </row>
-    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="19" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="B29" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C29" s="18"/>
-      <c r="D29" s="19" t="s">
+    <row r="27" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="20" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B30" s="18" t="s">
+      <c r="B27" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="C27" s="21"/>
+      <c r="D27" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="C30" s="18"/>
-      <c r="D30" s="19" t="s">
-        <v>79</v>
+      <c r="B28" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="21"/>
+      <c r="D28" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" s="21"/>
+      <c r="D29" s="12" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="B31" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="C31" s="18"/>
-      <c r="D31" s="19" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="B32" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="C32" s="18"/>
-      <c r="D32" s="19" t="s">
+      <c r="A31" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B32" s="21" t="s">
         <v>85</v>
       </c>
+      <c r="C32" s="21"/>
+      <c r="D32" s="13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+    </row>
+    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C36" s="18"/>
+      <c r="D36" s="19" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C37" s="18"/>
+      <c r="D37" s="19" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C38" s="18"/>
+      <c r="D38" s="19" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="C39" s="18"/>
+      <c r="D39" s="19" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="C40" s="18"/>
+      <c r="D40" s="19" t="s">
+        <v>103</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
     <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1857,22 +2016,22 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="2" style="0" width="5.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="2" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1884,6 +2043,10 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -1899,61 +2062,81 @@
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="C5" s="23"/>
-      <c r="D5" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24" t="s">
-        <v>91</v>
-      </c>
+      <c r="D5" s="23"/>
+      <c r="E5" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="F5" s="24"/>
       <c r="G5" s="24"/>
       <c r="H5" s="24" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="L5" s="24"/>
+      <c r="M5" s="24"/>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="H6" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="I6" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="J6" s="25" t="s">
-        <v>101</v>
+        <v>116</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>119</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>70</v>
+        <v>120</v>
+      </c>
+      <c r="L6" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="M6" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="N6" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1962,19 +2145,23 @@
       </c>
       <c r="B7" s="26"/>
       <c r="C7" s="26"/>
-      <c r="D7" s="15" t="s">
-        <v>102</v>
-      </c>
+      <c r="D7" s="26"/>
       <c r="E7" s="26"/>
       <c r="F7" s="26"/>
       <c r="G7" s="26"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="J7" s="27"/>
-      <c r="K7" s="10" t="s">
-        <v>104</v>
+      <c r="H7" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="27"/>
+      <c r="M7" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="N7" s="27"/>
+      <c r="O7" s="10" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1985,57 +2172,71 @@
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
       <c r="E8" s="26"/>
-      <c r="F8" s="15" t="s">
-        <v>105</v>
-      </c>
+      <c r="F8" s="26"/>
       <c r="G8" s="26"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="K8" s="10" t="s">
-        <v>106</v>
+      <c r="H8" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="N8" s="27"/>
+      <c r="O8" s="10" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>16</v>
+      <c r="A9" s="8" t="s">
+        <v>14</v>
       </c>
       <c r="B9" s="26"/>
       <c r="C9" s="26"/>
       <c r="D9" s="26"/>
       <c r="E9" s="26"/>
       <c r="F9" s="26"/>
-      <c r="G9" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H9" s="27"/>
-      <c r="I9" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="J9" s="27"/>
-      <c r="K9" s="10" t="s">
-        <v>107</v>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="K9" s="26"/>
+      <c r="L9" s="27"/>
+      <c r="M9" s="27"/>
+      <c r="N9" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="O9" s="10" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>102</v>
-      </c>
+      <c r="B10" s="26"/>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
       <c r="E10" s="26"/>
       <c r="F10" s="26"/>
       <c r="G10" s="26"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="10" t="s">
-        <v>108</v>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="L10" s="27"/>
+      <c r="M10" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="N10" s="27"/>
+      <c r="O10" s="10" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2043,165 +2244,205 @@
         <v>16</v>
       </c>
       <c r="B11" s="26"/>
-      <c r="C11" s="14" t="s">
-        <v>103</v>
-      </c>
+      <c r="C11" s="26"/>
       <c r="D11" s="26"/>
       <c r="E11" s="26"/>
       <c r="F11" s="15" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="G11" s="26"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="10" t="s">
-        <v>110</v>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="26"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="27"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="10" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
-        <v>18</v>
+      <c r="A12" s="11" t="s">
+        <v>16</v>
       </c>
       <c r="B12" s="26"/>
       <c r="C12" s="26"/>
       <c r="D12" s="26"/>
-      <c r="E12" s="14" t="s">
-        <v>103</v>
-      </c>
+      <c r="E12" s="26"/>
       <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
-      <c r="K12" s="10" t="s">
-        <v>111</v>
+      <c r="G12" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
+      <c r="J12" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="K12" s="26"/>
+      <c r="L12" s="27"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="27"/>
+      <c r="O12" s="10" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="26"/>
+      <c r="B13" s="15" t="s">
+        <v>127</v>
+      </c>
       <c r="C13" s="26"/>
       <c r="D13" s="26"/>
       <c r="E13" s="26"/>
       <c r="F13" s="26"/>
       <c r="G13" s="26"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27"/>
-      <c r="K13" s="10" t="s">
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
+      <c r="K13" s="26"/>
+      <c r="L13" s="27"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="27"/>
+      <c r="O13" s="10" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="J14" s="26"/>
+      <c r="K14" s="26"/>
+      <c r="L14" s="27"/>
+      <c r="M14" s="27"/>
+      <c r="N14" s="27"/>
+      <c r="O14" s="10" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="26"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+      <c r="O15" s="10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="6"/>
+      <c r="O17" s="6"/>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="B18" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="24" t="s">
+        <v>139</v>
+      </c>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="L18" s="24"/>
+      <c r="M18" s="24"/>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-    </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="B16" s="23" t="s">
+      <c r="D19" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23" t="s">
+      <c r="E19" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="E16" s="23"/>
-      <c r="F16" s="24" t="s">
+      <c r="F19" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24" t="s">
+      <c r="G19" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="I16" s="24"/>
-    </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="H17" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="I17" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="J17" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="K17" s="7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="14" t="s">
+      <c r="H19" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="J18" s="27"/>
-      <c r="K18" s="10" t="s">
+      <c r="I19" s="7" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="14" t="s">
+      <c r="J19" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
-      <c r="K19" s="10" t="s">
+      <c r="K19" s="7" t="s">
         <v>120</v>
+      </c>
+      <c r="L19" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="M19" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="N19" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="O19" s="7" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2214,22 +2455,22 @@
       <c r="E20" s="26"/>
       <c r="F20" s="26"/>
       <c r="G20" s="26"/>
-      <c r="H20" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="I20" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="J20" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="K20" s="10" t="s">
-        <v>123</v>
+      <c r="H20" s="26"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="27"/>
+      <c r="M20" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="N20" s="27"/>
+      <c r="O20" s="10" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>22</v>
+      <c r="A21" s="8" t="s">
+        <v>20</v>
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="26"/>
@@ -2237,63 +2478,71 @@
       <c r="E21" s="26"/>
       <c r="F21" s="26"/>
       <c r="G21" s="26"/>
-      <c r="H21" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="I21" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="J21" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="K21" s="10" t="s">
-        <v>125</v>
+      <c r="H21" s="26"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="10" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
-        <v>18</v>
+      <c r="A22" s="8" t="s">
+        <v>20</v>
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="26"/>
       <c r="D22" s="26"/>
       <c r="E22" s="26"/>
-      <c r="F22" s="14" t="s">
-        <v>117</v>
-      </c>
+      <c r="F22" s="26"/>
       <c r="G22" s="26"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="J22" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="K22" s="10" t="s">
-        <v>127</v>
+      <c r="H22" s="26"/>
+      <c r="I22" s="26"/>
+      <c r="J22" s="26"/>
+      <c r="K22" s="26"/>
+      <c r="L22" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="M22" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="N22" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="O22" s="10" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
-        <v>18</v>
+      <c r="A23" s="11" t="s">
+        <v>22</v>
       </c>
       <c r="B23" s="26"/>
       <c r="C23" s="26"/>
-      <c r="D23" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="F23" s="15" t="s">
-        <v>121</v>
-      </c>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
       <c r="G23" s="26"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="10" t="s">
-        <v>128</v>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="26"/>
+      <c r="L23" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="M23" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="N23" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="O23" s="10" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2306,40 +2555,102 @@
       <c r="E24" s="26"/>
       <c r="F24" s="26"/>
       <c r="G24" s="26"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="27"/>
-      <c r="J24" s="27"/>
-      <c r="K24" s="10" t="s">
-        <v>129</v>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="K24" s="26"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="N24" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="O24" s="10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" s="26"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="I25" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="K25" s="26"/>
+      <c r="L25" s="27"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="10" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
+      <c r="A26" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="26"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="26"/>
+      <c r="K26" s="26"/>
+      <c r="L26" s="27"/>
+      <c r="M26" s="27"/>
+      <c r="N26" s="27"/>
+      <c r="O26" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+      <c r="L28" s="2"/>
+      <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
+      <c r="O28" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="A28:O28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2384,12 +2695,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>131</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2415,7 +2726,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -2447,64 +2758,64 @@
         <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="T6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="V6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3147,7 +3458,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="31" t="n">
@@ -3203,7 +3514,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>146</v>
+        <v>170</v>
       </c>
       <c r="B18" s="18"/>
       <c r="C18" s="28"/>
@@ -3235,7 +3546,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>147</v>
+        <v>171</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="32" t="str">
@@ -3321,64 +3632,64 @@
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="N22" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="O22" s="7" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="Q22" s="7" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="R22" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="S22" s="7" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="T22" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="U22" s="7" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="V22" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3569,7 +3880,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="31" t="n">
@@ -3655,64 +3966,64 @@
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="N29" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="O29" s="7" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="P29" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="Q29" s="7" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="R29" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="S29" s="7" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="T29" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="U29" s="7" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="V29" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3903,7 +4214,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="31" t="n">
@@ -3959,7 +4270,7 @@
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -3985,73 +4296,73 @@
     </row>
     <row r="36" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>149</v>
+        <v>173</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="M36" s="7" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="N36" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="O36" s="7" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="P36" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="Q36" s="7" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="R36" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="S36" s="7" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="T36" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="U36" s="7" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="V36" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>150</v>
+        <v>174</v>
       </c>
       <c r="B37" s="12"/>
       <c r="C37" s="28"/>
@@ -4113,7 +4424,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="28"/>
@@ -4175,7 +4486,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>152</v>
+        <v>176</v>
       </c>
       <c r="B39" s="12"/>
       <c r="C39" s="28"/>
@@ -4237,7 +4548,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>153</v>
+        <v>177</v>
       </c>
       <c r="B40" s="12"/>
       <c r="C40" s="28"/>
@@ -4299,7 +4610,7 @@
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>154</v>
+        <v>178</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -4325,7 +4636,7 @@
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>155</v>
+        <v>179</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -4405,12 +4716,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>156</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>157</v>
+        <v>181</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4424,7 +4735,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -4444,28 +4755,28 @@
         <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>158</v>
+        <v>182</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="E6" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>135</v>
-      </c>
       <c r="G6" s="7" t="s">
-        <v>160</v>
+        <v>184</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>161</v>
+        <v>185</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4748,7 +5059,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="31" t="n">

</xml_diff>

<commit_message>
A2 travel rule (D-A2-15): Skip when UAE activity ends within 1 month of the last ticket and 1 month of silence; spec, model doc, v02 validation prompt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="196">
   <si>
     <t xml:space="preserve">A2 Locatability</t>
   </si>
@@ -77,7 +77,7 @@
     <t xml:space="preserve">Skip</t>
   </si>
   <si>
-    <t xml:space="preserve">The latest evidence places the customer abroad, however old it is.</t>
+    <t xml:space="preserve">The latest evidence places the customer abroad (however old), or they went silent soon after buying a ticket.</t>
   </si>
   <si>
     <t xml:space="preserve">Unknown</t>
@@ -194,22 +194,25 @@
     <t xml:space="preserve">Travel purchase</t>
   </si>
   <si>
-    <t xml:space="preserve">Airline, cruise or travel-agency purchase, dated on the purchase day.</t>
+    <t xml:space="preserve">Airline, cruise or travel-agency purchase, any channel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Departure signal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any date (travel rule)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collector note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer left the country (final exit visa included).</t>
   </si>
   <si>
     <t xml:space="preserve">Foreign</t>
   </si>
   <si>
-    <t xml:space="preserve">12 months; older ones are ignored</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collector note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer left the country (final exit visa included).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A travel purchase is foreign evidence like any other: it gives Skip unless UAE evidence comes after it (the customer came back or never left).</t>
+    <t xml:space="preserve">A ticket is bought weeks before the flight and the customer stays active until then, so a ticket is not compared with UAE activity by date: it feeds the travel rule (Location, rule 2).</t>
   </si>
   <si>
     <t xml:space="preserve">Features</t>
@@ -230,7 +233,13 @@
     <t xml:space="preserve">Latest foreign evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Most recent date of foreign evidence, travel purchases included while under 12 months old.</t>
+    <t xml:space="preserve">Most recent date of foreign evidence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last travel purchase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most recent date of a travel purchase.</t>
   </si>
   <si>
     <t xml:space="preserve">Last contact</t>
@@ -263,10 +272,16 @@
     <t xml:space="preserve">Rule 2</t>
   </si>
   <si>
+    <t xml:space="preserve">Travel rule: the latest UAE evidence is at most 1 month after the last travel purchase (or there is none), and no UAE evidence for at least 1 month since.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rule 3</t>
+  </si>
+  <si>
     <t xml:space="preserve">The latest evidence is UAE evidence within the window.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rule 3</t>
+    <t xml:space="preserve">Rule 4</t>
   </si>
   <si>
     <t xml:space="preserve">Otherwise: no evidence at all, or the latest UAE evidence is older than the window.</t>
@@ -314,10 +329,22 @@
     <t xml:space="preserve">No sign of return means still abroad.</t>
   </si>
   <si>
-    <t xml:space="preserve">Counts for 12 months.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">An old ticket says little about today.</t>
+    <t xml:space="preserve">Travel rule: gap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UAE activity ends at most 1 month after the ticket.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tickets are bought days to weeks before the flight.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel rule: silence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At least 1 month without UAE evidence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keeps a customer who just bought a ticket and is still active out of Skip.</t>
   </si>
   <si>
     <t xml:space="preserve">Failed call days</t>
@@ -407,16 +434,22 @@
     <t xml:space="preserve">Abroad 6 months ago; card used in the UAE last month.</t>
   </si>
   <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collector noted a departure; UAE login since.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bought a flight this month and still active: not silent yet.</t>
+  </si>
+  <si>
     <t xml:space="preserve">T</t>
   </si>
   <si>
-    <t xml:space="preserve">Flight bought, then card used in the UAE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collector noted a departure; UAE login since.</t>
+    <t xml:space="preserve">Flight bought, active for months after: back or never left.</t>
   </si>
   <si>
     <t xml:space="preserve">Latest login is from abroad.</t>
@@ -425,13 +458,10 @@
     <t xml:space="preserve">Last seen abroad 8 months ago, nothing since.</t>
   </si>
   <si>
-    <t xml:space="preserve">Flight bought 4 months ago, no UAE activity since.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only a flight bought 12 months ago: too old, ignored.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last UAE activity is older than the window.</t>
+    <t xml:space="preserve">Flight bought, UAE activity stopped a month later, silent since.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active long after the flight, then quiet beyond the window.</t>
   </si>
   <si>
     <t xml:space="preserve">No evidence at all.</t>
@@ -1592,7 +1622,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -1664,7 +1694,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
         <v>55</v>
       </c>
@@ -1686,7 +1716,7 @@
         <v>60</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D9" s="19" t="s">
         <v>51</v>
@@ -1694,7 +1724,7 @@
     </row>
     <row r="10" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1702,7 +1732,7 @@
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -1710,10 +1740,10 @@
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7" t="s">
@@ -1722,22 +1752,22 @@
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C14" s="18"/>
       <c r="D14" s="19" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C15" s="18"/>
       <c r="D15" s="19" t="s">
@@ -1746,22 +1776,22 @@
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C16" s="18"/>
       <c r="D16" s="19" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C17" s="18"/>
       <c r="D17" s="19" t="s">
@@ -1770,179 +1800,179 @@
     </row>
     <row r="18" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="19" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="18"/>
+      <c r="D19" s="19" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-    </row>
-    <row r="22" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="B22" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="C22" s="21"/>
-      <c r="D22" s="11" t="s">
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+    </row>
+    <row r="23" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="21"/>
+      <c r="D23" s="11" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="C23" s="21"/>
-      <c r="D23" s="8" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B24" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="21"/>
+      <c r="D24" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="21"/>
+      <c r="D25" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="C26" s="21"/>
+      <c r="D26" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+    </row>
+    <row r="29" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="21"/>
+      <c r="D29" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="12" t="s">
+      <c r="B30" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" s="21"/>
+      <c r="D30" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" s="21"/>
+      <c r="D31" s="12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-    </row>
-    <row r="27" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="B27" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="C27" s="21"/>
-      <c r="D27" s="11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="B28" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C28" s="21"/>
-      <c r="D28" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C29" s="21"/>
-      <c r="D29" s="12" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
+    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-    </row>
-    <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="B32" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="C32" s="21"/>
-      <c r="D32" s="13" t="s">
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="C34" s="21"/>
+      <c r="D34" s="13" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-    </row>
-    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B36" s="18" t="s">
+    <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="C36" s="18"/>
-      <c r="D36" s="19" t="s">
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+    </row>
+    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17" t="s">
+      <c r="B37" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B37" s="18" t="s">
+      <c r="C37" s="7"/>
+      <c r="D37" s="7" t="s">
         <v>94</v>
-      </c>
-      <c r="C37" s="18"/>
-      <c r="D37" s="19" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="17" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="B38" s="18" t="s">
         <v>96</v>
@@ -1952,7 +1982,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
         <v>98</v>
       </c>
@@ -1976,8 +2006,44 @@
         <v>103</v>
       </c>
     </row>
+    <row r="41" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="C41" s="18"/>
+      <c r="D41" s="19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" s="18"/>
+      <c r="D42" s="19" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="C43" s="18"/>
+      <c r="D43" s="19" t="s">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="25">
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="B13:C13"/>
@@ -1986,20 +2052,23 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="A20:D20"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2026,12 +2095,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2069,25 +2138,25 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="C5" s="23"/>
       <c r="D5" s="23"/>
       <c r="E5" s="24" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="F5" s="24"/>
       <c r="G5" s="24"/>
       <c r="H5" s="24" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="I5" s="24"/>
       <c r="J5" s="24"/>
       <c r="K5" s="24" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="L5" s="24"/>
       <c r="M5" s="24"/>
@@ -2097,46 +2166,46 @@
         <v>11</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="L6" s="25" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="N6" s="25" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2150,18 +2219,18 @@
       <c r="F7" s="26"/>
       <c r="G7" s="26"/>
       <c r="H7" s="15" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="I7" s="26"/>
       <c r="J7" s="26"/>
       <c r="K7" s="26"/>
       <c r="L7" s="27"/>
       <c r="M7" s="14" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="N7" s="27"/>
       <c r="O7" s="10" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2174,19 +2243,19 @@
       <c r="E8" s="26"/>
       <c r="F8" s="26"/>
       <c r="G8" s="26"/>
-      <c r="H8" s="15" t="s">
-        <v>127</v>
-      </c>
+      <c r="H8" s="26"/>
       <c r="I8" s="26"/>
-      <c r="J8" s="26"/>
+      <c r="J8" s="15" t="s">
+        <v>136</v>
+      </c>
       <c r="K8" s="26"/>
       <c r="L8" s="27"/>
-      <c r="M8" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="N8" s="27"/>
+      <c r="M8" s="27"/>
+      <c r="N8" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="O8" s="10" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2201,42 +2270,42 @@
       <c r="G9" s="26"/>
       <c r="H9" s="26"/>
       <c r="I9" s="26"/>
-      <c r="J9" s="15" t="s">
-        <v>129</v>
-      </c>
+      <c r="J9" s="26"/>
       <c r="K9" s="26"/>
       <c r="L9" s="27"/>
       <c r="M9" s="27"/>
       <c r="N9" s="14" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>16</v>
+      <c r="A10" s="8" t="s">
+        <v>14</v>
       </c>
       <c r="B10" s="26"/>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
       <c r="E10" s="26"/>
       <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
+      <c r="G10" s="15" t="s">
+        <v>140</v>
+      </c>
       <c r="H10" s="26"/>
       <c r="I10" s="26"/>
       <c r="J10" s="26"/>
       <c r="K10" s="14" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="L10" s="27"/>
-      <c r="M10" s="15" t="s">
-        <v>124</v>
+      <c r="M10" s="14" t="s">
+        <v>134</v>
       </c>
       <c r="N10" s="27"/>
       <c r="O10" s="10" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2247,19 +2316,21 @@
       <c r="C11" s="26"/>
       <c r="D11" s="26"/>
       <c r="E11" s="26"/>
-      <c r="F11" s="15" t="s">
-        <v>124</v>
-      </c>
+      <c r="F11" s="26"/>
       <c r="G11" s="26"/>
       <c r="H11" s="26"/>
       <c r="I11" s="26"/>
       <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
+      <c r="K11" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="L11" s="27"/>
-      <c r="M11" s="27"/>
+      <c r="M11" s="15" t="s">
+        <v>133</v>
+      </c>
       <c r="N11" s="27"/>
       <c r="O11" s="10" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2270,30 +2341,26 @@
       <c r="C12" s="26"/>
       <c r="D12" s="26"/>
       <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="14" t="s">
-        <v>125</v>
-      </c>
+      <c r="F12" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="G12" s="26"/>
       <c r="H12" s="26"/>
       <c r="I12" s="26"/>
-      <c r="J12" s="15" t="s">
-        <v>127</v>
-      </c>
+      <c r="J12" s="26"/>
       <c r="K12" s="26"/>
       <c r="L12" s="27"/>
       <c r="M12" s="27"/>
       <c r="N12" s="27"/>
       <c r="O12" s="10" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>127</v>
-      </c>
+      <c r="A13" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="26"/>
       <c r="C13" s="26"/>
       <c r="D13" s="26"/>
       <c r="E13" s="26"/>
@@ -2303,11 +2370,15 @@
       <c r="I13" s="26"/>
       <c r="J13" s="26"/>
       <c r="K13" s="26"/>
-      <c r="L13" s="27"/>
-      <c r="M13" s="27"/>
+      <c r="L13" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="M13" s="14" t="s">
+        <v>134</v>
+      </c>
       <c r="N13" s="27"/>
       <c r="O13" s="10" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2316,13 +2387,15 @@
       </c>
       <c r="B14" s="26"/>
       <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
+      <c r="D14" s="15" t="s">
+        <v>140</v>
+      </c>
       <c r="E14" s="26"/>
       <c r="F14" s="26"/>
       <c r="G14" s="26"/>
       <c r="H14" s="26"/>
       <c r="I14" s="14" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="J14" s="26"/>
       <c r="K14" s="26"/>
@@ -2330,7 +2403,7 @@
       <c r="M14" s="27"/>
       <c r="N14" s="27"/>
       <c r="O14" s="10" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2351,7 +2424,7 @@
       <c r="M15" s="27"/>
       <c r="N15" s="27"/>
       <c r="O15" s="10" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2375,25 +2448,25 @@
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="C18" s="23"/>
       <c r="D18" s="23"/>
       <c r="E18" s="23" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="F18" s="23"/>
       <c r="G18" s="23"/>
       <c r="H18" s="24" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="I18" s="24"/>
       <c r="J18" s="24"/>
       <c r="K18" s="24" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="L18" s="24"/>
       <c r="M18" s="24"/>
@@ -2403,46 +2476,46 @@
         <v>11</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="L19" s="25" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="M19" s="25" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="N19" s="25" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2461,11 +2534,11 @@
       <c r="K20" s="26"/>
       <c r="L20" s="27"/>
       <c r="M20" s="14" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="N20" s="27"/>
       <c r="O20" s="10" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2483,12 +2556,12 @@
       <c r="J21" s="26"/>
       <c r="K21" s="26"/>
       <c r="L21" s="14" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="M21" s="27"/>
       <c r="N21" s="27"/>
       <c r="O21" s="10" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2506,16 +2579,16 @@
       <c r="J22" s="26"/>
       <c r="K22" s="26"/>
       <c r="L22" s="15" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="M22" s="15" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="N22" s="14" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="O22" s="10" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2533,16 +2606,16 @@
       <c r="J23" s="26"/>
       <c r="K23" s="26"/>
       <c r="L23" s="14" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="M23" s="15" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="N23" s="15" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2558,18 +2631,18 @@
       <c r="H24" s="26"/>
       <c r="I24" s="26"/>
       <c r="J24" s="14" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="K24" s="26"/>
       <c r="L24" s="27"/>
       <c r="M24" s="15" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="N24" s="15" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="O24" s="10" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2583,20 +2656,20 @@
       <c r="F25" s="26"/>
       <c r="G25" s="26"/>
       <c r="H25" s="15" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="J25" s="15" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="K25" s="26"/>
       <c r="L25" s="27"/>
       <c r="M25" s="27"/>
       <c r="N25" s="27"/>
       <c r="O25" s="10" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2617,12 +2690,12 @@
       <c r="M26" s="27"/>
       <c r="N26" s="27"/>
       <c r="O26" s="10" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -2695,12 +2768,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2726,7 +2799,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -2758,64 +2831,64 @@
         <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="T6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="V6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3458,7 +3531,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="31" t="n">
@@ -3514,7 +3587,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="B18" s="18"/>
       <c r="C18" s="28"/>
@@ -3546,7 +3619,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="32" t="str">
@@ -3632,64 +3705,64 @@
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="N22" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="O22" s="7" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="Q22" s="7" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="R22" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="S22" s="7" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="T22" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="U22" s="7" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="V22" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3880,7 +3953,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="31" t="n">
@@ -3966,64 +4039,64 @@
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="N29" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="O29" s="7" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="P29" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="Q29" s="7" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="R29" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="S29" s="7" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="T29" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="U29" s="7" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="V29" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4214,7 +4287,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="31" t="n">
@@ -4270,7 +4343,7 @@
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -4296,73 +4369,73 @@
     </row>
     <row r="36" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="M36" s="7" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="N36" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="O36" s="7" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="P36" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="Q36" s="7" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="R36" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="S36" s="7" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="T36" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="U36" s="7" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="V36" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="B37" s="12"/>
       <c r="C37" s="28"/>
@@ -4424,7 +4497,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="28"/>
@@ -4486,7 +4559,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B39" s="12"/>
       <c r="C39" s="28"/>
@@ -4548,7 +4621,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="B40" s="12"/>
       <c r="C40" s="28"/>
@@ -4610,7 +4683,7 @@
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -4636,7 +4709,7 @@
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -4716,12 +4789,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4735,7 +4808,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -4755,28 +4828,28 @@
         <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5059,7 +5132,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="31" t="n">

</xml_diff>

<commit_message>
A2 model doc: explicit Evidence table (event -> UAE / foreign evidence, departure signal, contact, failed call day, deceased); features defined on it
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="192">
   <si>
     <t xml:space="preserve">A2 Locatability</t>
   </si>
@@ -155,64 +155,58 @@
     <t xml:space="preserve">What the model computes for each account at the scoring date, and the rules that turn it into states. Within a dimension, the first rule that holds decides.</t>
   </si>
   <si>
-    <t xml:space="preserve">Location evidence</t>
-  </si>
-  <si>
     <t xml:space="preserve">Evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">What counts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UAE or foreign</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Counts for</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Digital-banking login.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">By login country</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Any date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Card use</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In-person card use (shop payment, ATM withdrawal) on any of the customer's cards and accounts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">By where it was used</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Travel purchase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Airline, cruise or travel-agency purchase, any channel.</t>
+    <t xml:space="preserve">Event</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Counts as</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login from the UAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UAE evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shop payment or ATM withdrawal in the UAE, in person, on any of the customer's cards and accounts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login from abroad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foreign evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shop payment or ATM withdrawal abroad, in person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collector note: customer left the country (final exit visa included)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel purchase (airline, cruise, travel agency), any channel</t>
   </si>
   <si>
     <t xml:space="preserve">Departure signal</t>
   </si>
   <si>
-    <t xml:space="preserve">Any date (travel rule)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collector note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer left the country (final exit visa included).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Foreign</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A ticket is bought weeks before the flight and the customer stays active until then, so a ticket is not compared with UAE activity by date: it feeds the travel rule (Location, rule 2).</t>
+    <t xml:space="preserve">Customer answered our call, or called us</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A day we called and every call rang out or hit a dead line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failed call day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collector note of death (claims included), card blocked as deceased, or customer record marked deceased</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every event is dated and counts at any age; the rules decide how recent it must be. A ticket is bought weeks before the flight, so it is not compared with UAE activity by date: it is used only by the travel rule (Location, rule 2). Ignored: logins with no country, online purchases, transfers and remittances, salary.</t>
   </si>
   <si>
     <t xml:space="preserve">Features</t>
@@ -227,40 +221,37 @@
     <t xml:space="preserve">Latest UAE evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Most recent date of UAE evidence.</t>
+    <t xml:space="preserve">Date of the most recent UAE evidence.</t>
   </si>
   <si>
     <t xml:space="preserve">Latest foreign evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Most recent date of foreign evidence.</t>
+    <t xml:space="preserve">Date of the most recent foreign evidence.</t>
   </si>
   <si>
     <t xml:space="preserve">Last travel purchase</t>
   </si>
   <si>
-    <t xml:space="preserve">Most recent date of a travel purchase.</t>
+    <t xml:space="preserve">Date of the most recent departure signal.</t>
   </si>
   <si>
     <t xml:space="preserve">Last contact</t>
   </si>
   <si>
-    <t xml:space="preserve">Date of the most recent day the customer answered our call or called us.</t>
+    <t xml:space="preserve">Date of the most recent contact.</t>
   </si>
   <si>
     <t xml:space="preserve">Last 3 call days</t>
   </si>
   <si>
-    <t xml:space="preserve">Outcome of the 3 most recent days we called. A day fails when every call rang out or hit a dead line.</t>
+    <t xml:space="preserve">The 3 most recent days we called, each failed or not.</t>
   </si>
   <si>
     <t xml:space="preserve">Deceased flag</t>
   </si>
   <si>
-    <t xml:space="preserve">Collector note of death (claims included), card blocked as deceased, or customer record marked deceased.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not used: online purchases, transfers and remittances (they do not show where the customer is), and salary (an ability signal).</t>
+    <t xml:space="preserve">Any deceased evidence, at any date.</t>
   </si>
   <si>
     <t xml:space="preserve">Rule 1</t>
@@ -318,9 +309,6 @@
   </si>
   <si>
     <t xml:space="preserve">Same as the other axes; activity is thinner at 180+.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Foreign evidence</t>
   </si>
   <si>
     <t xml:space="preserve">No age limit.</t>
@@ -900,7 +888,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -970,6 +958,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -979,14 +979,6 @@
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1622,7 +1614,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -1656,419 +1648,470 @@
       <c r="A5" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="B6" s="10"/>
+      <c r="C6" s="8" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
+      <c r="D6" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B7" s="10"/>
+      <c r="C7" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="B8" s="10"/>
+      <c r="C8" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D8" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
+      <c r="B9" s="10"/>
+      <c r="C9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B10" s="10"/>
+      <c r="C10" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="B11" s="10"/>
+      <c r="C11" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D7" s="19" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
+      <c r="D11" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B12" s="10"/>
+      <c r="C12" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="D12" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="B13" s="10"/>
+      <c r="C13" s="11" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
+      <c r="D13" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B14" s="10"/>
+      <c r="C14" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D9" s="19" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="B18" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-    </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+      <c r="C18" s="7"/>
+      <c r="D18" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B19" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
+      <c r="C19" s="10"/>
+      <c r="D19" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B20" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="19" t="s">
+      <c r="C20" s="10"/>
+      <c r="D20" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B21" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="19" t="s">
+      <c r="C21" s="10"/>
+      <c r="D21" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
+    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B22" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="19" t="s">
+      <c r="C22" s="10"/>
+      <c r="D22" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" s="10"/>
+      <c r="D23" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="10"/>
+      <c r="D24" s="9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="19" t="s">
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+    </row>
+    <row r="27" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" s="19"/>
+      <c r="D27" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="19"/>
+      <c r="D28" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" s="19"/>
+      <c r="D29" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" s="19"/>
+      <c r="D30" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="B18" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C18" s="18"/>
-      <c r="D18" s="19" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+    </row>
+    <row r="33" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="B19" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="C19" s="18"/>
-      <c r="D19" s="19" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="B33" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C33" s="19"/>
+      <c r="D33" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-    </row>
-    <row r="23" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="B23" s="21" t="s">
+      <c r="B34" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34" s="19"/>
+      <c r="D34" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="C23" s="21"/>
-      <c r="D23" s="11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="B25" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="B26" s="21" t="s">
+      <c r="B35" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="C26" s="21"/>
-      <c r="D26" s="12" t="s">
+      <c r="C35" s="19"/>
+      <c r="D35" s="12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-    </row>
-    <row r="29" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="B29" s="21" t="s">
+    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+    </row>
+    <row r="38" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="B38" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="C29" s="21"/>
-      <c r="D29" s="11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="B30" s="21" t="s">
+      <c r="C38" s="19"/>
+      <c r="D38" s="13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C30" s="21"/>
-      <c r="D30" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="B31" s="21" t="s">
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+    </row>
+    <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C31" s="21"/>
-      <c r="D31" s="12" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-    </row>
-    <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="B34" s="21" t="s">
+      <c r="B41" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C34" s="21"/>
-      <c r="D34" s="13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
+      <c r="C41" s="7"/>
+      <c r="D41" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-    </row>
-    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
+    </row>
+    <row r="42" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B37" s="7" t="s">
+      <c r="B42" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7" t="s">
+      <c r="C42" s="21"/>
+      <c r="D42" s="22" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17" t="s">
+    <row r="43" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B43" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="B38" s="18" t="s">
+      <c r="C43" s="21"/>
+      <c r="D43" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="C38" s="18"/>
-      <c r="D38" s="19" t="s">
+    </row>
+    <row r="44" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="20" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17" t="s">
+      <c r="B44" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="B39" s="18" t="s">
+      <c r="C44" s="21"/>
+      <c r="D44" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="C39" s="18"/>
-      <c r="D39" s="19" t="s">
+    </row>
+    <row r="45" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="20" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17" t="s">
+      <c r="B45" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="B40" s="18" t="s">
+      <c r="C45" s="21"/>
+      <c r="D45" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="C40" s="18"/>
-      <c r="D40" s="19" t="s">
+    </row>
+    <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="20" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="41" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17" t="s">
+      <c r="B46" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="B41" s="18" t="s">
+      <c r="C46" s="21"/>
+      <c r="D46" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="C41" s="18"/>
-      <c r="D41" s="19" t="s">
+    </row>
+    <row r="47" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="20" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17" t="s">
+      <c r="B47" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="B42" s="18" t="s">
+      <c r="C47" s="21"/>
+      <c r="D47" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="C42" s="18"/>
-      <c r="D42" s="19" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="B43" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="C43" s="18"/>
-      <c r="D43" s="19" t="s">
-        <v>112</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="34">
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:D15"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B19:C19"/>
-    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2095,12 +2138,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2137,294 +2180,294 @@
       <c r="O4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="I5" s="25"/>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25" t="s">
         <v>115</v>
       </c>
-      <c r="B5" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="I5" s="24"/>
-      <c r="J5" s="24"/>
-      <c r="K5" s="24" t="s">
-        <v>119</v>
-      </c>
-      <c r="L5" s="24"/>
-      <c r="M5" s="24"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="25"/>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="I6" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="J6" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="K6" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="L6" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="M6" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="N6" s="26" t="s">
         <v>128</v>
       </c>
-      <c r="K6" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="L6" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="M6" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="N6" s="25" t="s">
-        <v>132</v>
-      </c>
       <c r="O6" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
       <c r="H7" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="I7" s="26"/>
-      <c r="J7" s="26"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="27"/>
+        <v>129</v>
+      </c>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="28"/>
       <c r="M7" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="N7" s="27"/>
+        <v>130</v>
+      </c>
+      <c r="N7" s="28"/>
       <c r="O7" s="10" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
       <c r="J8" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="K8" s="26"/>
-      <c r="L8" s="27"/>
-      <c r="M8" s="27"/>
+        <v>132</v>
+      </c>
+      <c r="K8" s="27"/>
+      <c r="L8" s="28"/>
+      <c r="M8" s="28"/>
       <c r="N8" s="14" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="26"/>
-      <c r="K9" s="26"/>
-      <c r="L9" s="27"/>
-      <c r="M9" s="27"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="27"/>
+      <c r="L9" s="28"/>
+      <c r="M9" s="28"/>
       <c r="N9" s="14" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
       <c r="G10" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
+        <v>136</v>
+      </c>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
       <c r="K10" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="L10" s="27"/>
+        <v>130</v>
+      </c>
+      <c r="L10" s="28"/>
       <c r="M10" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="N10" s="27"/>
+        <v>130</v>
+      </c>
+      <c r="N10" s="28"/>
       <c r="O10" s="10" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="26"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
       <c r="K11" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="L11" s="27"/>
+        <v>130</v>
+      </c>
+      <c r="L11" s="28"/>
       <c r="M11" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="N11" s="27"/>
+        <v>129</v>
+      </c>
+      <c r="N11" s="28"/>
       <c r="O11" s="10" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
       <c r="F12" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="27"/>
-      <c r="M12" s="27"/>
-      <c r="N12" s="27"/>
+        <v>129</v>
+      </c>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="28"/>
+      <c r="M12" s="28"/>
+      <c r="N12" s="28"/>
       <c r="O12" s="10" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="26"/>
-      <c r="K13" s="26"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
+      <c r="K13" s="27"/>
       <c r="L13" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="M13" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="N13" s="28"/>
+      <c r="O13" s="10" t="s">
         <v>140</v>
-      </c>
-      <c r="M13" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="N13" s="27"/>
-      <c r="O13" s="10" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="27"/>
       <c r="D14" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
+        <v>136</v>
+      </c>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
       <c r="I14" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="J14" s="26"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="27"/>
-      <c r="M14" s="27"/>
-      <c r="N14" s="27"/>
+        <v>130</v>
+      </c>
+      <c r="J14" s="27"/>
+      <c r="K14" s="27"/>
+      <c r="L14" s="28"/>
+      <c r="M14" s="28"/>
+      <c r="N14" s="28"/>
       <c r="O14" s="10" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="26"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="27"/>
-      <c r="M15" s="27"/>
-      <c r="N15" s="27"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="28"/>
+      <c r="M15" s="28"/>
+      <c r="N15" s="28"/>
       <c r="O15" s="10" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2447,255 +2490,255 @@
       <c r="O17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="24" t="s">
-        <v>149</v>
-      </c>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="24" t="s">
-        <v>150</v>
-      </c>
-      <c r="L18" s="24"/>
-      <c r="M18" s="24"/>
+      <c r="A18" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="B18" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="I18" s="25"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="L18" s="25"/>
+      <c r="M18" s="25"/>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B19" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="F19" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="G19" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="H19" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="I19" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="J19" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="K19" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="L19" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="M19" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="J19" s="7" t="s">
+      <c r="N19" s="26" t="s">
         <v>128</v>
       </c>
-      <c r="K19" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="L19" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="M19" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="N19" s="25" t="s">
-        <v>132</v>
-      </c>
       <c r="O19" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="26"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="26"/>
-      <c r="K20" s="26"/>
-      <c r="L20" s="27"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="28"/>
       <c r="M20" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="N20" s="27"/>
+        <v>147</v>
+      </c>
+      <c r="N20" s="28"/>
       <c r="O20" s="10" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="26"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
       <c r="L21" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="M21" s="27"/>
-      <c r="N21" s="27"/>
+        <v>149</v>
+      </c>
+      <c r="M21" s="28"/>
+      <c r="N21" s="28"/>
       <c r="O21" s="10" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="26"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="26"/>
-      <c r="K22" s="26"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
       <c r="L22" s="15" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="M22" s="15" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="N22" s="14" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="O22" s="10" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26"/>
-      <c r="I23" s="26"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="26"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
       <c r="L23" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="M23" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="N23" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="M23" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="N23" s="15" t="s">
+      <c r="O23" s="10" t="s">
         <v>155</v>
-      </c>
-      <c r="O23" s="10" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="26"/>
-      <c r="I24" s="26"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
       <c r="J24" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="K24" s="27"/>
+      <c r="L24" s="28"/>
+      <c r="M24" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="K24" s="26"/>
-      <c r="L24" s="27"/>
-      <c r="M24" s="15" t="s">
-        <v>155</v>
-      </c>
       <c r="N24" s="15" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="O24" s="10" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
       <c r="H25" s="15" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="J25" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="K25" s="26"/>
-      <c r="L25" s="27"/>
-      <c r="M25" s="27"/>
-      <c r="N25" s="27"/>
+        <v>151</v>
+      </c>
+      <c r="K25" s="27"/>
+      <c r="L25" s="28"/>
+      <c r="M25" s="28"/>
+      <c r="N25" s="28"/>
       <c r="O25" s="10" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B26" s="26"/>
-      <c r="C26" s="26"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="26"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="26"/>
-      <c r="L26" s="27"/>
-      <c r="M26" s="27"/>
-      <c r="N26" s="27"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
+      <c r="I26" s="27"/>
+      <c r="J26" s="27"/>
+      <c r="K26" s="27"/>
+      <c r="L26" s="28"/>
+      <c r="M26" s="28"/>
+      <c r="N26" s="28"/>
       <c r="O26" s="10" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -2768,12 +2811,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2799,7 +2842,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -2831,64 +2874,64 @@
         <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="I6" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="J6" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="K6" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="L6" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="M6" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="G6" s="7" t="s">
+      <c r="N6" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="O6" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="I6" s="7" t="s">
+      <c r="P6" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q6" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="J6" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="K6" s="7" t="s">
+      <c r="R6" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="S6" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="L6" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="M6" s="7" t="s">
+      <c r="T6" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="U6" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="N6" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="Q6" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="R6" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="S6" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="T6" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="U6" s="7" t="s">
-        <v>178</v>
-      </c>
       <c r="V6" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2896,59 +2939,59 @@
         <v>25</v>
       </c>
       <c r="B7" s="13"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="29" t="str">
+      <c r="C7" s="29"/>
+      <c r="D7" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C7/$C$17)</f>
         <v/>
       </c>
-      <c r="E7" s="28"/>
-      <c r="F7" s="29" t="str">
+      <c r="E7" s="29"/>
+      <c r="F7" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E7/$E$17)</f>
         <v/>
       </c>
-      <c r="G7" s="28"/>
-      <c r="H7" s="29" t="str">
+      <c r="G7" s="29"/>
+      <c r="H7" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G7/$G$17)</f>
         <v/>
       </c>
-      <c r="I7" s="28"/>
-      <c r="J7" s="29" t="str">
+      <c r="I7" s="29"/>
+      <c r="J7" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I7/$I$17)</f>
         <v/>
       </c>
-      <c r="K7" s="28"/>
-      <c r="L7" s="29" t="str">
+      <c r="K7" s="29"/>
+      <c r="L7" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K7/$K$17)</f>
         <v/>
       </c>
-      <c r="M7" s="30" t="n">
+      <c r="M7" s="31" t="n">
         <f aca="false">G7+I7+K7</f>
         <v>0</v>
       </c>
-      <c r="N7" s="29" t="str">
+      <c r="N7" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M7/$M$17)</f>
         <v/>
       </c>
-      <c r="O7" s="28"/>
-      <c r="P7" s="29" t="str">
+      <c r="O7" s="29"/>
+      <c r="P7" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O7/$O$17)</f>
         <v/>
       </c>
-      <c r="Q7" s="28"/>
-      <c r="R7" s="29" t="str">
+      <c r="Q7" s="29"/>
+      <c r="R7" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q7/$Q$17)</f>
         <v/>
       </c>
-      <c r="S7" s="28"/>
-      <c r="T7" s="29" t="str">
+      <c r="S7" s="29"/>
+      <c r="T7" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S7/$S$17)</f>
         <v/>
       </c>
-      <c r="U7" s="30" t="n">
+      <c r="U7" s="31" t="n">
         <f aca="false">O7+Q7+S7</f>
         <v>0</v>
       </c>
-      <c r="V7" s="29" t="str">
+      <c r="V7" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U7/$U$17)</f>
         <v/>
       </c>
@@ -2960,59 +3003,59 @@
       <c r="B8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="29" t="str">
+      <c r="C8" s="29"/>
+      <c r="D8" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C8/$C$17)</f>
         <v/>
       </c>
-      <c r="E8" s="28"/>
-      <c r="F8" s="29" t="str">
+      <c r="E8" s="29"/>
+      <c r="F8" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E8/$E$17)</f>
         <v/>
       </c>
-      <c r="G8" s="28"/>
-      <c r="H8" s="29" t="str">
+      <c r="G8" s="29"/>
+      <c r="H8" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G8/$G$17)</f>
         <v/>
       </c>
-      <c r="I8" s="28"/>
-      <c r="J8" s="29" t="str">
+      <c r="I8" s="29"/>
+      <c r="J8" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I8/$I$17)</f>
         <v/>
       </c>
-      <c r="K8" s="28"/>
-      <c r="L8" s="29" t="str">
+      <c r="K8" s="29"/>
+      <c r="L8" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K8/$K$17)</f>
         <v/>
       </c>
-      <c r="M8" s="30" t="n">
+      <c r="M8" s="31" t="n">
         <f aca="false">G8+I8+K8</f>
         <v>0</v>
       </c>
-      <c r="N8" s="29" t="str">
+      <c r="N8" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M8/$M$17)</f>
         <v/>
       </c>
-      <c r="O8" s="28"/>
-      <c r="P8" s="29" t="str">
+      <c r="O8" s="29"/>
+      <c r="P8" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O8/$O$17)</f>
         <v/>
       </c>
-      <c r="Q8" s="28"/>
-      <c r="R8" s="29" t="str">
+      <c r="Q8" s="29"/>
+      <c r="R8" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q8/$Q$17)</f>
         <v/>
       </c>
-      <c r="S8" s="28"/>
-      <c r="T8" s="29" t="str">
+      <c r="S8" s="29"/>
+      <c r="T8" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S8/$S$17)</f>
         <v/>
       </c>
-      <c r="U8" s="30" t="n">
+      <c r="U8" s="31" t="n">
         <f aca="false">O8+Q8+S8</f>
         <v>0</v>
       </c>
-      <c r="V8" s="29" t="str">
+      <c r="V8" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U8/$U$17)</f>
         <v/>
       </c>
@@ -3024,59 +3067,59 @@
       <c r="B9" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="29" t="str">
+      <c r="C9" s="29"/>
+      <c r="D9" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C9/$C$17)</f>
         <v/>
       </c>
-      <c r="E9" s="28"/>
-      <c r="F9" s="29" t="str">
+      <c r="E9" s="29"/>
+      <c r="F9" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E9/$E$17)</f>
         <v/>
       </c>
-      <c r="G9" s="28"/>
-      <c r="H9" s="29" t="str">
+      <c r="G9" s="29"/>
+      <c r="H9" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G9/$G$17)</f>
         <v/>
       </c>
-      <c r="I9" s="28"/>
-      <c r="J9" s="29" t="str">
+      <c r="I9" s="29"/>
+      <c r="J9" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I9/$I$17)</f>
         <v/>
       </c>
-      <c r="K9" s="28"/>
-      <c r="L9" s="29" t="str">
+      <c r="K9" s="29"/>
+      <c r="L9" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K9/$K$17)</f>
         <v/>
       </c>
-      <c r="M9" s="30" t="n">
+      <c r="M9" s="31" t="n">
         <f aca="false">G9+I9+K9</f>
         <v>0</v>
       </c>
-      <c r="N9" s="29" t="str">
+      <c r="N9" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M9/$M$17)</f>
         <v/>
       </c>
-      <c r="O9" s="28"/>
-      <c r="P9" s="29" t="str">
+      <c r="O9" s="29"/>
+      <c r="P9" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O9/$O$17)</f>
         <v/>
       </c>
-      <c r="Q9" s="28"/>
-      <c r="R9" s="29" t="str">
+      <c r="Q9" s="29"/>
+      <c r="R9" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q9/$Q$17)</f>
         <v/>
       </c>
-      <c r="S9" s="28"/>
-      <c r="T9" s="29" t="str">
+      <c r="S9" s="29"/>
+      <c r="T9" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S9/$S$17)</f>
         <v/>
       </c>
-      <c r="U9" s="30" t="n">
+      <c r="U9" s="31" t="n">
         <f aca="false">O9+Q9+S9</f>
         <v>0</v>
       </c>
-      <c r="V9" s="29" t="str">
+      <c r="V9" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U9/$U$17)</f>
         <v/>
       </c>
@@ -3088,59 +3131,59 @@
       <c r="B10" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="29" t="str">
+      <c r="C10" s="29"/>
+      <c r="D10" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C10/$C$17)</f>
         <v/>
       </c>
-      <c r="E10" s="28"/>
-      <c r="F10" s="29" t="str">
+      <c r="E10" s="29"/>
+      <c r="F10" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E10/$E$17)</f>
         <v/>
       </c>
-      <c r="G10" s="28"/>
-      <c r="H10" s="29" t="str">
+      <c r="G10" s="29"/>
+      <c r="H10" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G10/$G$17)</f>
         <v/>
       </c>
-      <c r="I10" s="28"/>
-      <c r="J10" s="29" t="str">
+      <c r="I10" s="29"/>
+      <c r="J10" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I10/$I$17)</f>
         <v/>
       </c>
-      <c r="K10" s="28"/>
-      <c r="L10" s="29" t="str">
+      <c r="K10" s="29"/>
+      <c r="L10" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K10/$K$17)</f>
         <v/>
       </c>
-      <c r="M10" s="30" t="n">
+      <c r="M10" s="31" t="n">
         <f aca="false">G10+I10+K10</f>
         <v>0</v>
       </c>
-      <c r="N10" s="29" t="str">
+      <c r="N10" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M10/$M$17)</f>
         <v/>
       </c>
-      <c r="O10" s="28"/>
-      <c r="P10" s="29" t="str">
+      <c r="O10" s="29"/>
+      <c r="P10" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O10/$O$17)</f>
         <v/>
       </c>
-      <c r="Q10" s="28"/>
-      <c r="R10" s="29" t="str">
+      <c r="Q10" s="29"/>
+      <c r="R10" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q10/$Q$17)</f>
         <v/>
       </c>
-      <c r="S10" s="28"/>
-      <c r="T10" s="29" t="str">
+      <c r="S10" s="29"/>
+      <c r="T10" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S10/$S$17)</f>
         <v/>
       </c>
-      <c r="U10" s="30" t="n">
+      <c r="U10" s="31" t="n">
         <f aca="false">O10+Q10+S10</f>
         <v>0</v>
       </c>
-      <c r="V10" s="29" t="str">
+      <c r="V10" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U10/$U$17)</f>
         <v/>
       </c>
@@ -3152,59 +3195,59 @@
       <c r="B11" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="28"/>
-      <c r="D11" s="29" t="str">
+      <c r="C11" s="29"/>
+      <c r="D11" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C11/$C$17)</f>
         <v/>
       </c>
-      <c r="E11" s="28"/>
-      <c r="F11" s="29" t="str">
+      <c r="E11" s="29"/>
+      <c r="F11" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E11/$E$17)</f>
         <v/>
       </c>
-      <c r="G11" s="28"/>
-      <c r="H11" s="29" t="str">
+      <c r="G11" s="29"/>
+      <c r="H11" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G11/$G$17)</f>
         <v/>
       </c>
-      <c r="I11" s="28"/>
-      <c r="J11" s="29" t="str">
+      <c r="I11" s="29"/>
+      <c r="J11" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I11/$I$17)</f>
         <v/>
       </c>
-      <c r="K11" s="28"/>
-      <c r="L11" s="29" t="str">
+      <c r="K11" s="29"/>
+      <c r="L11" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K11/$K$17)</f>
         <v/>
       </c>
-      <c r="M11" s="30" t="n">
+      <c r="M11" s="31" t="n">
         <f aca="false">G11+I11+K11</f>
         <v>0</v>
       </c>
-      <c r="N11" s="29" t="str">
+      <c r="N11" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M11/$M$17)</f>
         <v/>
       </c>
-      <c r="O11" s="28"/>
-      <c r="P11" s="29" t="str">
+      <c r="O11" s="29"/>
+      <c r="P11" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O11/$O$17)</f>
         <v/>
       </c>
-      <c r="Q11" s="28"/>
-      <c r="R11" s="29" t="str">
+      <c r="Q11" s="29"/>
+      <c r="R11" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q11/$Q$17)</f>
         <v/>
       </c>
-      <c r="S11" s="28"/>
-      <c r="T11" s="29" t="str">
+      <c r="S11" s="29"/>
+      <c r="T11" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S11/$S$17)</f>
         <v/>
       </c>
-      <c r="U11" s="30" t="n">
+      <c r="U11" s="31" t="n">
         <f aca="false">O11+Q11+S11</f>
         <v>0</v>
       </c>
-      <c r="V11" s="29" t="str">
+      <c r="V11" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U11/$U$17)</f>
         <v/>
       </c>
@@ -3216,59 +3259,59 @@
       <c r="B12" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="29" t="str">
+      <c r="C12" s="29"/>
+      <c r="D12" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C12/$C$17)</f>
         <v/>
       </c>
-      <c r="E12" s="28"/>
-      <c r="F12" s="29" t="str">
+      <c r="E12" s="29"/>
+      <c r="F12" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E12/$E$17)</f>
         <v/>
       </c>
-      <c r="G12" s="28"/>
-      <c r="H12" s="29" t="str">
+      <c r="G12" s="29"/>
+      <c r="H12" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G12/$G$17)</f>
         <v/>
       </c>
-      <c r="I12" s="28"/>
-      <c r="J12" s="29" t="str">
+      <c r="I12" s="29"/>
+      <c r="J12" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I12/$I$17)</f>
         <v/>
       </c>
-      <c r="K12" s="28"/>
-      <c r="L12" s="29" t="str">
+      <c r="K12" s="29"/>
+      <c r="L12" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K12/$K$17)</f>
         <v/>
       </c>
-      <c r="M12" s="30" t="n">
+      <c r="M12" s="31" t="n">
         <f aca="false">G12+I12+K12</f>
         <v>0</v>
       </c>
-      <c r="N12" s="29" t="str">
+      <c r="N12" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M12/$M$17)</f>
         <v/>
       </c>
-      <c r="O12" s="28"/>
-      <c r="P12" s="29" t="str">
+      <c r="O12" s="29"/>
+      <c r="P12" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O12/$O$17)</f>
         <v/>
       </c>
-      <c r="Q12" s="28"/>
-      <c r="R12" s="29" t="str">
+      <c r="Q12" s="29"/>
+      <c r="R12" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q12/$Q$17)</f>
         <v/>
       </c>
-      <c r="S12" s="28"/>
-      <c r="T12" s="29" t="str">
+      <c r="S12" s="29"/>
+      <c r="T12" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S12/$S$17)</f>
         <v/>
       </c>
-      <c r="U12" s="30" t="n">
+      <c r="U12" s="31" t="n">
         <f aca="false">O12+Q12+S12</f>
         <v>0</v>
       </c>
-      <c r="V12" s="29" t="str">
+      <c r="V12" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U12/$U$17)</f>
         <v/>
       </c>
@@ -3280,59 +3323,59 @@
       <c r="B13" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="28"/>
-      <c r="D13" s="29" t="str">
+      <c r="C13" s="29"/>
+      <c r="D13" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C13/$C$17)</f>
         <v/>
       </c>
-      <c r="E13" s="28"/>
-      <c r="F13" s="29" t="str">
+      <c r="E13" s="29"/>
+      <c r="F13" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E13/$E$17)</f>
         <v/>
       </c>
-      <c r="G13" s="28"/>
-      <c r="H13" s="29" t="str">
+      <c r="G13" s="29"/>
+      <c r="H13" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G13/$G$17)</f>
         <v/>
       </c>
-      <c r="I13" s="28"/>
-      <c r="J13" s="29" t="str">
+      <c r="I13" s="29"/>
+      <c r="J13" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I13/$I$17)</f>
         <v/>
       </c>
-      <c r="K13" s="28"/>
-      <c r="L13" s="29" t="str">
+      <c r="K13" s="29"/>
+      <c r="L13" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K13/$K$17)</f>
         <v/>
       </c>
-      <c r="M13" s="30" t="n">
+      <c r="M13" s="31" t="n">
         <f aca="false">G13+I13+K13</f>
         <v>0</v>
       </c>
-      <c r="N13" s="29" t="str">
+      <c r="N13" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M13/$M$17)</f>
         <v/>
       </c>
-      <c r="O13" s="28"/>
-      <c r="P13" s="29" t="str">
+      <c r="O13" s="29"/>
+      <c r="P13" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O13/$O$17)</f>
         <v/>
       </c>
-      <c r="Q13" s="28"/>
-      <c r="R13" s="29" t="str">
+      <c r="Q13" s="29"/>
+      <c r="R13" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q13/$Q$17)</f>
         <v/>
       </c>
-      <c r="S13" s="28"/>
-      <c r="T13" s="29" t="str">
+      <c r="S13" s="29"/>
+      <c r="T13" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S13/$S$17)</f>
         <v/>
       </c>
-      <c r="U13" s="30" t="n">
+      <c r="U13" s="31" t="n">
         <f aca="false">O13+Q13+S13</f>
         <v>0</v>
       </c>
-      <c r="V13" s="29" t="str">
+      <c r="V13" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U13/$U$17)</f>
         <v/>
       </c>
@@ -3344,59 +3387,59 @@
       <c r="B14" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="29" t="str">
+      <c r="C14" s="29"/>
+      <c r="D14" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C14/$C$17)</f>
         <v/>
       </c>
-      <c r="E14" s="28"/>
-      <c r="F14" s="29" t="str">
+      <c r="E14" s="29"/>
+      <c r="F14" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E14/$E$17)</f>
         <v/>
       </c>
-      <c r="G14" s="28"/>
-      <c r="H14" s="29" t="str">
+      <c r="G14" s="29"/>
+      <c r="H14" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G14/$G$17)</f>
         <v/>
       </c>
-      <c r="I14" s="28"/>
-      <c r="J14" s="29" t="str">
+      <c r="I14" s="29"/>
+      <c r="J14" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I14/$I$17)</f>
         <v/>
       </c>
-      <c r="K14" s="28"/>
-      <c r="L14" s="29" t="str">
+      <c r="K14" s="29"/>
+      <c r="L14" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K14/$K$17)</f>
         <v/>
       </c>
-      <c r="M14" s="30" t="n">
+      <c r="M14" s="31" t="n">
         <f aca="false">G14+I14+K14</f>
         <v>0</v>
       </c>
-      <c r="N14" s="29" t="str">
+      <c r="N14" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M14/$M$17)</f>
         <v/>
       </c>
-      <c r="O14" s="28"/>
-      <c r="P14" s="29" t="str">
+      <c r="O14" s="29"/>
+      <c r="P14" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O14/$O$17)</f>
         <v/>
       </c>
-      <c r="Q14" s="28"/>
-      <c r="R14" s="29" t="str">
+      <c r="Q14" s="29"/>
+      <c r="R14" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q14/$Q$17)</f>
         <v/>
       </c>
-      <c r="S14" s="28"/>
-      <c r="T14" s="29" t="str">
+      <c r="S14" s="29"/>
+      <c r="T14" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S14/$S$17)</f>
         <v/>
       </c>
-      <c r="U14" s="30" t="n">
+      <c r="U14" s="31" t="n">
         <f aca="false">O14+Q14+S14</f>
         <v>0</v>
       </c>
-      <c r="V14" s="29" t="str">
+      <c r="V14" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U14/$U$17)</f>
         <v/>
       </c>
@@ -3408,59 +3451,59 @@
       <c r="B15" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="29" t="str">
+      <c r="C15" s="29"/>
+      <c r="D15" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C15/$C$17)</f>
         <v/>
       </c>
-      <c r="E15" s="28"/>
-      <c r="F15" s="29" t="str">
+      <c r="E15" s="29"/>
+      <c r="F15" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E15/$E$17)</f>
         <v/>
       </c>
-      <c r="G15" s="28"/>
-      <c r="H15" s="29" t="str">
+      <c r="G15" s="29"/>
+      <c r="H15" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G15/$G$17)</f>
         <v/>
       </c>
-      <c r="I15" s="28"/>
-      <c r="J15" s="29" t="str">
+      <c r="I15" s="29"/>
+      <c r="J15" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I15/$I$17)</f>
         <v/>
       </c>
-      <c r="K15" s="28"/>
-      <c r="L15" s="29" t="str">
+      <c r="K15" s="29"/>
+      <c r="L15" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K15/$K$17)</f>
         <v/>
       </c>
-      <c r="M15" s="30" t="n">
+      <c r="M15" s="31" t="n">
         <f aca="false">G15+I15+K15</f>
         <v>0</v>
       </c>
-      <c r="N15" s="29" t="str">
+      <c r="N15" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M15/$M$17)</f>
         <v/>
       </c>
-      <c r="O15" s="28"/>
-      <c r="P15" s="29" t="str">
+      <c r="O15" s="29"/>
+      <c r="P15" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O15/$O$17)</f>
         <v/>
       </c>
-      <c r="Q15" s="28"/>
-      <c r="R15" s="29" t="str">
+      <c r="Q15" s="29"/>
+      <c r="R15" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q15/$Q$17)</f>
         <v/>
       </c>
-      <c r="S15" s="28"/>
-      <c r="T15" s="29" t="str">
+      <c r="S15" s="29"/>
+      <c r="T15" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S15/$S$17)</f>
         <v/>
       </c>
-      <c r="U15" s="30" t="n">
+      <c r="U15" s="31" t="n">
         <f aca="false">O15+Q15+S15</f>
         <v>0</v>
       </c>
-      <c r="V15" s="29" t="str">
+      <c r="V15" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U15/$U$17)</f>
         <v/>
       </c>
@@ -3472,206 +3515,206 @@
       <c r="B16" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="28"/>
-      <c r="D16" s="29" t="str">
+      <c r="C16" s="29"/>
+      <c r="D16" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C16/$C$17)</f>
         <v/>
       </c>
-      <c r="E16" s="28"/>
-      <c r="F16" s="29" t="str">
+      <c r="E16" s="29"/>
+      <c r="F16" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E16/$E$17)</f>
         <v/>
       </c>
-      <c r="G16" s="28"/>
-      <c r="H16" s="29" t="str">
+      <c r="G16" s="29"/>
+      <c r="H16" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G16/$G$17)</f>
         <v/>
       </c>
-      <c r="I16" s="28"/>
-      <c r="J16" s="29" t="str">
+      <c r="I16" s="29"/>
+      <c r="J16" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I16/$I$17)</f>
         <v/>
       </c>
-      <c r="K16" s="28"/>
-      <c r="L16" s="29" t="str">
+      <c r="K16" s="29"/>
+      <c r="L16" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K16/$K$17)</f>
         <v/>
       </c>
-      <c r="M16" s="30" t="n">
+      <c r="M16" s="31" t="n">
         <f aca="false">G16+I16+K16</f>
         <v>0</v>
       </c>
-      <c r="N16" s="29" t="str">
+      <c r="N16" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M16/$M$17)</f>
         <v/>
       </c>
-      <c r="O16" s="28"/>
-      <c r="P16" s="29" t="str">
+      <c r="O16" s="29"/>
+      <c r="P16" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O16/$O$17)</f>
         <v/>
       </c>
-      <c r="Q16" s="28"/>
-      <c r="R16" s="29" t="str">
+      <c r="Q16" s="29"/>
+      <c r="R16" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q16/$Q$17)</f>
         <v/>
       </c>
-      <c r="S16" s="28"/>
-      <c r="T16" s="29" t="str">
+      <c r="S16" s="29"/>
+      <c r="T16" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S16/$S$17)</f>
         <v/>
       </c>
-      <c r="U16" s="30" t="n">
+      <c r="U16" s="31" t="n">
         <f aca="false">O16+Q16+S16</f>
         <v>0</v>
       </c>
-      <c r="V16" s="29" t="str">
+      <c r="V16" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U16/$U$17)</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="31" t="n">
+      <c r="A17" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="B17" s="20"/>
+      <c r="C17" s="32" t="n">
         <f aca="false">SUM(C7:C16)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="18"/>
-      <c r="E17" s="31" t="n">
+      <c r="D17" s="21"/>
+      <c r="E17" s="32" t="n">
         <f aca="false">SUM(E7:E16)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="18"/>
-      <c r="G17" s="31" t="n">
+      <c r="F17" s="21"/>
+      <c r="G17" s="32" t="n">
         <f aca="false">SUM(G7:G16)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="18"/>
-      <c r="I17" s="31" t="n">
+      <c r="H17" s="21"/>
+      <c r="I17" s="32" t="n">
         <f aca="false">SUM(I7:I16)</f>
         <v>0</v>
       </c>
-      <c r="J17" s="18"/>
-      <c r="K17" s="31" t="n">
+      <c r="J17" s="21"/>
+      <c r="K17" s="32" t="n">
         <f aca="false">SUM(K7:K16)</f>
         <v>0</v>
       </c>
-      <c r="L17" s="18"/>
-      <c r="M17" s="31" t="n">
+      <c r="L17" s="21"/>
+      <c r="M17" s="32" t="n">
         <f aca="false">SUM(M7:M16)</f>
         <v>0</v>
       </c>
-      <c r="N17" s="18"/>
-      <c r="O17" s="31" t="n">
+      <c r="N17" s="21"/>
+      <c r="O17" s="32" t="n">
         <f aca="false">SUM(O7:O16)</f>
         <v>0</v>
       </c>
-      <c r="P17" s="18"/>
-      <c r="Q17" s="31" t="n">
+      <c r="P17" s="21"/>
+      <c r="Q17" s="32" t="n">
         <f aca="false">SUM(Q7:Q16)</f>
         <v>0</v>
       </c>
-      <c r="R17" s="18"/>
-      <c r="S17" s="31" t="n">
+      <c r="R17" s="21"/>
+      <c r="S17" s="32" t="n">
         <f aca="false">SUM(S7:S16)</f>
         <v>0</v>
       </c>
-      <c r="T17" s="18"/>
-      <c r="U17" s="31" t="n">
+      <c r="T17" s="21"/>
+      <c r="U17" s="32" t="n">
         <f aca="false">SUM(U7:U16)</f>
         <v>0</v>
       </c>
-      <c r="V17" s="18"/>
+      <c r="V17" s="21"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
-        <v>180</v>
-      </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="28"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="30" t="n">
+      <c r="A18" s="21" t="s">
+        <v>176</v>
+      </c>
+      <c r="B18" s="21"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="29"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="29"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="31" t="n">
         <f aca="false">G18+I18+K18</f>
         <v>0</v>
       </c>
-      <c r="N18" s="18"/>
-      <c r="O18" s="28"/>
-      <c r="P18" s="18"/>
-      <c r="Q18" s="28"/>
-      <c r="R18" s="18"/>
-      <c r="S18" s="28"/>
-      <c r="T18" s="18"/>
-      <c r="U18" s="30" t="n">
+      <c r="N18" s="21"/>
+      <c r="O18" s="29"/>
+      <c r="P18" s="21"/>
+      <c r="Q18" s="29"/>
+      <c r="R18" s="21"/>
+      <c r="S18" s="29"/>
+      <c r="T18" s="21"/>
+      <c r="U18" s="31" t="n">
         <f aca="false">O18+Q18+S18</f>
         <v>0</v>
       </c>
-      <c r="V18" s="18"/>
+      <c r="V18" s="21"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="32" t="str">
+      <c r="A19" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="B19" s="20"/>
+      <c r="C19" s="33" t="str">
         <f aca="false">IF(C18=0,"",C17/C18)</f>
         <v/>
       </c>
-      <c r="D19" s="18"/>
-      <c r="E19" s="32" t="str">
+      <c r="D19" s="21"/>
+      <c r="E19" s="33" t="str">
         <f aca="false">IF(E18=0,"",E17/E18)</f>
         <v/>
       </c>
-      <c r="F19" s="18"/>
-      <c r="G19" s="32" t="str">
+      <c r="F19" s="21"/>
+      <c r="G19" s="33" t="str">
         <f aca="false">IF(G18=0,"",G17/G18)</f>
         <v/>
       </c>
-      <c r="H19" s="18"/>
-      <c r="I19" s="32" t="str">
+      <c r="H19" s="21"/>
+      <c r="I19" s="33" t="str">
         <f aca="false">IF(I18=0,"",I17/I18)</f>
         <v/>
       </c>
-      <c r="J19" s="18"/>
-      <c r="K19" s="32" t="str">
+      <c r="J19" s="21"/>
+      <c r="K19" s="33" t="str">
         <f aca="false">IF(K18=0,"",K17/K18)</f>
         <v/>
       </c>
-      <c r="L19" s="18"/>
-      <c r="M19" s="32" t="str">
+      <c r="L19" s="21"/>
+      <c r="M19" s="33" t="str">
         <f aca="false">IF(M18=0,"",M17/M18)</f>
         <v/>
       </c>
-      <c r="N19" s="18"/>
-      <c r="O19" s="32" t="str">
+      <c r="N19" s="21"/>
+      <c r="O19" s="33" t="str">
         <f aca="false">IF(O18=0,"",O17/O18)</f>
         <v/>
       </c>
-      <c r="P19" s="18"/>
-      <c r="Q19" s="32" t="str">
+      <c r="P19" s="21"/>
+      <c r="Q19" s="33" t="str">
         <f aca="false">IF(Q18=0,"",Q17/Q18)</f>
         <v/>
       </c>
-      <c r="R19" s="18"/>
-      <c r="S19" s="32" t="str">
+      <c r="R19" s="21"/>
+      <c r="S19" s="33" t="str">
         <f aca="false">IF(S18=0,"",S17/S18)</f>
         <v/>
       </c>
-      <c r="T19" s="18"/>
-      <c r="U19" s="32" t="str">
+      <c r="T19" s="21"/>
+      <c r="U19" s="33" t="str">
         <f aca="false">IF(U18=0,"",U17/U18)</f>
         <v/>
       </c>
-      <c r="V19" s="18"/>
+      <c r="V19" s="21"/>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
@@ -3705,64 +3748,64 @@
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="I22" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="J22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="K22" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="L22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="M22" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="G22" s="7" t="s">
+      <c r="N22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="O22" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="H22" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="I22" s="7" t="s">
+      <c r="P22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q22" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="J22" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="K22" s="7" t="s">
+      <c r="R22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="S22" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="L22" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="M22" s="7" t="s">
+      <c r="T22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="U22" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="N22" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="O22" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="P22" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="Q22" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="R22" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="S22" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="T22" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="U22" s="7" t="s">
-        <v>178</v>
-      </c>
       <c r="V22" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3770,59 +3813,59 @@
         <v>14</v>
       </c>
       <c r="B23" s="8"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="29" t="str">
+      <c r="C23" s="29"/>
+      <c r="D23" s="30" t="str">
         <f aca="false">IF($C$26=0,"",C23/$C$26)</f>
         <v/>
       </c>
-      <c r="E23" s="28"/>
-      <c r="F23" s="29" t="str">
+      <c r="E23" s="29"/>
+      <c r="F23" s="30" t="str">
         <f aca="false">IF($E$26=0,"",E23/$E$26)</f>
         <v/>
       </c>
-      <c r="G23" s="28"/>
-      <c r="H23" s="29" t="str">
+      <c r="G23" s="29"/>
+      <c r="H23" s="30" t="str">
         <f aca="false">IF($G$26=0,"",G23/$G$26)</f>
         <v/>
       </c>
-      <c r="I23" s="28"/>
-      <c r="J23" s="29" t="str">
+      <c r="I23" s="29"/>
+      <c r="J23" s="30" t="str">
         <f aca="false">IF($I$26=0,"",I23/$I$26)</f>
         <v/>
       </c>
-      <c r="K23" s="28"/>
-      <c r="L23" s="29" t="str">
+      <c r="K23" s="29"/>
+      <c r="L23" s="30" t="str">
         <f aca="false">IF($K$26=0,"",K23/$K$26)</f>
         <v/>
       </c>
-      <c r="M23" s="30" t="n">
+      <c r="M23" s="31" t="n">
         <f aca="false">G23+I23+K23</f>
         <v>0</v>
       </c>
-      <c r="N23" s="29" t="str">
+      <c r="N23" s="30" t="str">
         <f aca="false">IF($M$26=0,"",M23/$M$26)</f>
         <v/>
       </c>
-      <c r="O23" s="28"/>
-      <c r="P23" s="29" t="str">
+      <c r="O23" s="29"/>
+      <c r="P23" s="30" t="str">
         <f aca="false">IF($O$26=0,"",O23/$O$26)</f>
         <v/>
       </c>
-      <c r="Q23" s="28"/>
-      <c r="R23" s="29" t="str">
+      <c r="Q23" s="29"/>
+      <c r="R23" s="30" t="str">
         <f aca="false">IF($Q$26=0,"",Q23/$Q$26)</f>
         <v/>
       </c>
-      <c r="S23" s="28"/>
-      <c r="T23" s="29" t="str">
+      <c r="S23" s="29"/>
+      <c r="T23" s="30" t="str">
         <f aca="false">IF($S$26=0,"",S23/$S$26)</f>
         <v/>
       </c>
-      <c r="U23" s="30" t="n">
+      <c r="U23" s="31" t="n">
         <f aca="false">O23+Q23+S23</f>
         <v>0</v>
       </c>
-      <c r="V23" s="29" t="str">
+      <c r="V23" s="30" t="str">
         <f aca="false">IF($U$26=0,"",U23/$U$26)</f>
         <v/>
       </c>
@@ -3832,59 +3875,59 @@
         <v>16</v>
       </c>
       <c r="B24" s="11"/>
-      <c r="C24" s="28"/>
-      <c r="D24" s="29" t="str">
+      <c r="C24" s="29"/>
+      <c r="D24" s="30" t="str">
         <f aca="false">IF($C$26=0,"",C24/$C$26)</f>
         <v/>
       </c>
-      <c r="E24" s="28"/>
-      <c r="F24" s="29" t="str">
+      <c r="E24" s="29"/>
+      <c r="F24" s="30" t="str">
         <f aca="false">IF($E$26=0,"",E24/$E$26)</f>
         <v/>
       </c>
-      <c r="G24" s="28"/>
-      <c r="H24" s="29" t="str">
+      <c r="G24" s="29"/>
+      <c r="H24" s="30" t="str">
         <f aca="false">IF($G$26=0,"",G24/$G$26)</f>
         <v/>
       </c>
-      <c r="I24" s="28"/>
-      <c r="J24" s="29" t="str">
+      <c r="I24" s="29"/>
+      <c r="J24" s="30" t="str">
         <f aca="false">IF($I$26=0,"",I24/$I$26)</f>
         <v/>
       </c>
-      <c r="K24" s="28"/>
-      <c r="L24" s="29" t="str">
+      <c r="K24" s="29"/>
+      <c r="L24" s="30" t="str">
         <f aca="false">IF($K$26=0,"",K24/$K$26)</f>
         <v/>
       </c>
-      <c r="M24" s="30" t="n">
+      <c r="M24" s="31" t="n">
         <f aca="false">G24+I24+K24</f>
         <v>0</v>
       </c>
-      <c r="N24" s="29" t="str">
+      <c r="N24" s="30" t="str">
         <f aca="false">IF($M$26=0,"",M24/$M$26)</f>
         <v/>
       </c>
-      <c r="O24" s="28"/>
-      <c r="P24" s="29" t="str">
+      <c r="O24" s="29"/>
+      <c r="P24" s="30" t="str">
         <f aca="false">IF($O$26=0,"",O24/$O$26)</f>
         <v/>
       </c>
-      <c r="Q24" s="28"/>
-      <c r="R24" s="29" t="str">
+      <c r="Q24" s="29"/>
+      <c r="R24" s="30" t="str">
         <f aca="false">IF($Q$26=0,"",Q24/$Q$26)</f>
         <v/>
       </c>
-      <c r="S24" s="28"/>
-      <c r="T24" s="29" t="str">
+      <c r="S24" s="29"/>
+      <c r="T24" s="30" t="str">
         <f aca="false">IF($S$26=0,"",S24/$S$26)</f>
         <v/>
       </c>
-      <c r="U24" s="30" t="n">
+      <c r="U24" s="31" t="n">
         <f aca="false">O24+Q24+S24</f>
         <v>0</v>
       </c>
-      <c r="V24" s="29" t="str">
+      <c r="V24" s="30" t="str">
         <f aca="false">IF($U$26=0,"",U24/$U$26)</f>
         <v/>
       </c>
@@ -3894,118 +3937,118 @@
         <v>18</v>
       </c>
       <c r="B25" s="12"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="29" t="str">
+      <c r="C25" s="29"/>
+      <c r="D25" s="30" t="str">
         <f aca="false">IF($C$26=0,"",C25/$C$26)</f>
         <v/>
       </c>
-      <c r="E25" s="28"/>
-      <c r="F25" s="29" t="str">
+      <c r="E25" s="29"/>
+      <c r="F25" s="30" t="str">
         <f aca="false">IF($E$26=0,"",E25/$E$26)</f>
         <v/>
       </c>
-      <c r="G25" s="28"/>
-      <c r="H25" s="29" t="str">
+      <c r="G25" s="29"/>
+      <c r="H25" s="30" t="str">
         <f aca="false">IF($G$26=0,"",G25/$G$26)</f>
         <v/>
       </c>
-      <c r="I25" s="28"/>
-      <c r="J25" s="29" t="str">
+      <c r="I25" s="29"/>
+      <c r="J25" s="30" t="str">
         <f aca="false">IF($I$26=0,"",I25/$I$26)</f>
         <v/>
       </c>
-      <c r="K25" s="28"/>
-      <c r="L25" s="29" t="str">
+      <c r="K25" s="29"/>
+      <c r="L25" s="30" t="str">
         <f aca="false">IF($K$26=0,"",K25/$K$26)</f>
         <v/>
       </c>
-      <c r="M25" s="30" t="n">
+      <c r="M25" s="31" t="n">
         <f aca="false">G25+I25+K25</f>
         <v>0</v>
       </c>
-      <c r="N25" s="29" t="str">
+      <c r="N25" s="30" t="str">
         <f aca="false">IF($M$26=0,"",M25/$M$26)</f>
         <v/>
       </c>
-      <c r="O25" s="28"/>
-      <c r="P25" s="29" t="str">
+      <c r="O25" s="29"/>
+      <c r="P25" s="30" t="str">
         <f aca="false">IF($O$26=0,"",O25/$O$26)</f>
         <v/>
       </c>
-      <c r="Q25" s="28"/>
-      <c r="R25" s="29" t="str">
+      <c r="Q25" s="29"/>
+      <c r="R25" s="30" t="str">
         <f aca="false">IF($Q$26=0,"",Q25/$Q$26)</f>
         <v/>
       </c>
-      <c r="S25" s="28"/>
-      <c r="T25" s="29" t="str">
+      <c r="S25" s="29"/>
+      <c r="T25" s="30" t="str">
         <f aca="false">IF($S$26=0,"",S25/$S$26)</f>
         <v/>
       </c>
-      <c r="U25" s="30" t="n">
+      <c r="U25" s="31" t="n">
         <f aca="false">O25+Q25+S25</f>
         <v>0</v>
       </c>
-      <c r="V25" s="29" t="str">
+      <c r="V25" s="30" t="str">
         <f aca="false">IF($U$26=0,"",U25/$U$26)</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="31" t="n">
+      <c r="A26" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="B26" s="20"/>
+      <c r="C26" s="32" t="n">
         <f aca="false">SUM(C23:C25)</f>
         <v>0</v>
       </c>
-      <c r="D26" s="18"/>
-      <c r="E26" s="31" t="n">
+      <c r="D26" s="21"/>
+      <c r="E26" s="32" t="n">
         <f aca="false">SUM(E23:E25)</f>
         <v>0</v>
       </c>
-      <c r="F26" s="18"/>
-      <c r="G26" s="31" t="n">
+      <c r="F26" s="21"/>
+      <c r="G26" s="32" t="n">
         <f aca="false">SUM(G23:G25)</f>
         <v>0</v>
       </c>
-      <c r="H26" s="18"/>
-      <c r="I26" s="31" t="n">
+      <c r="H26" s="21"/>
+      <c r="I26" s="32" t="n">
         <f aca="false">SUM(I23:I25)</f>
         <v>0</v>
       </c>
-      <c r="J26" s="18"/>
-      <c r="K26" s="31" t="n">
+      <c r="J26" s="21"/>
+      <c r="K26" s="32" t="n">
         <f aca="false">SUM(K23:K25)</f>
         <v>0</v>
       </c>
-      <c r="L26" s="18"/>
-      <c r="M26" s="31" t="n">
+      <c r="L26" s="21"/>
+      <c r="M26" s="32" t="n">
         <f aca="false">SUM(M23:M25)</f>
         <v>0</v>
       </c>
-      <c r="N26" s="18"/>
-      <c r="O26" s="31" t="n">
+      <c r="N26" s="21"/>
+      <c r="O26" s="32" t="n">
         <f aca="false">SUM(O23:O25)</f>
         <v>0</v>
       </c>
-      <c r="P26" s="18"/>
-      <c r="Q26" s="31" t="n">
+      <c r="P26" s="21"/>
+      <c r="Q26" s="32" t="n">
         <f aca="false">SUM(Q23:Q25)</f>
         <v>0</v>
       </c>
-      <c r="R26" s="18"/>
-      <c r="S26" s="31" t="n">
+      <c r="R26" s="21"/>
+      <c r="S26" s="32" t="n">
         <f aca="false">SUM(S23:S25)</f>
         <v>0</v>
       </c>
-      <c r="T26" s="18"/>
-      <c r="U26" s="31" t="n">
+      <c r="T26" s="21"/>
+      <c r="U26" s="32" t="n">
         <f aca="false">SUM(U23:U25)</f>
         <v>0</v>
       </c>
-      <c r="V26" s="18"/>
+      <c r="V26" s="21"/>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
@@ -4039,64 +4082,64 @@
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="I29" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="J29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="K29" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="L29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="M29" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="G29" s="7" t="s">
+      <c r="N29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="O29" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="H29" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="I29" s="7" t="s">
+      <c r="P29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q29" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="J29" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="K29" s="7" t="s">
+      <c r="R29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="S29" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="L29" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="M29" s="7" t="s">
+      <c r="T29" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="U29" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="N29" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="O29" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="P29" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="Q29" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="R29" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="S29" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="T29" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="U29" s="7" t="s">
-        <v>178</v>
-      </c>
       <c r="V29" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4104,59 +4147,59 @@
         <v>20</v>
       </c>
       <c r="B30" s="8"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="29" t="str">
+      <c r="C30" s="29"/>
+      <c r="D30" s="30" t="str">
         <f aca="false">IF($C$33=0,"",C30/$C$33)</f>
         <v/>
       </c>
-      <c r="E30" s="28"/>
-      <c r="F30" s="29" t="str">
+      <c r="E30" s="29"/>
+      <c r="F30" s="30" t="str">
         <f aca="false">IF($E$33=0,"",E30/$E$33)</f>
         <v/>
       </c>
-      <c r="G30" s="28"/>
-      <c r="H30" s="29" t="str">
+      <c r="G30" s="29"/>
+      <c r="H30" s="30" t="str">
         <f aca="false">IF($G$33=0,"",G30/$G$33)</f>
         <v/>
       </c>
-      <c r="I30" s="28"/>
-      <c r="J30" s="29" t="str">
+      <c r="I30" s="29"/>
+      <c r="J30" s="30" t="str">
         <f aca="false">IF($I$33=0,"",I30/$I$33)</f>
         <v/>
       </c>
-      <c r="K30" s="28"/>
-      <c r="L30" s="29" t="str">
+      <c r="K30" s="29"/>
+      <c r="L30" s="30" t="str">
         <f aca="false">IF($K$33=0,"",K30/$K$33)</f>
         <v/>
       </c>
-      <c r="M30" s="30" t="n">
+      <c r="M30" s="31" t="n">
         <f aca="false">G30+I30+K30</f>
         <v>0</v>
       </c>
-      <c r="N30" s="29" t="str">
+      <c r="N30" s="30" t="str">
         <f aca="false">IF($M$33=0,"",M30/$M$33)</f>
         <v/>
       </c>
-      <c r="O30" s="28"/>
-      <c r="P30" s="29" t="str">
+      <c r="O30" s="29"/>
+      <c r="P30" s="30" t="str">
         <f aca="false">IF($O$33=0,"",O30/$O$33)</f>
         <v/>
       </c>
-      <c r="Q30" s="28"/>
-      <c r="R30" s="29" t="str">
+      <c r="Q30" s="29"/>
+      <c r="R30" s="30" t="str">
         <f aca="false">IF($Q$33=0,"",Q30/$Q$33)</f>
         <v/>
       </c>
-      <c r="S30" s="28"/>
-      <c r="T30" s="29" t="str">
+      <c r="S30" s="29"/>
+      <c r="T30" s="30" t="str">
         <f aca="false">IF($S$33=0,"",S30/$S$33)</f>
         <v/>
       </c>
-      <c r="U30" s="30" t="n">
+      <c r="U30" s="31" t="n">
         <f aca="false">O30+Q30+S30</f>
         <v>0</v>
       </c>
-      <c r="V30" s="29" t="str">
+      <c r="V30" s="30" t="str">
         <f aca="false">IF($U$33=0,"",U30/$U$33)</f>
         <v/>
       </c>
@@ -4166,59 +4209,59 @@
         <v>22</v>
       </c>
       <c r="B31" s="11"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="29" t="str">
+      <c r="C31" s="29"/>
+      <c r="D31" s="30" t="str">
         <f aca="false">IF($C$33=0,"",C31/$C$33)</f>
         <v/>
       </c>
-      <c r="E31" s="28"/>
-      <c r="F31" s="29" t="str">
+      <c r="E31" s="29"/>
+      <c r="F31" s="30" t="str">
         <f aca="false">IF($E$33=0,"",E31/$E$33)</f>
         <v/>
       </c>
-      <c r="G31" s="28"/>
-      <c r="H31" s="29" t="str">
+      <c r="G31" s="29"/>
+      <c r="H31" s="30" t="str">
         <f aca="false">IF($G$33=0,"",G31/$G$33)</f>
         <v/>
       </c>
-      <c r="I31" s="28"/>
-      <c r="J31" s="29" t="str">
+      <c r="I31" s="29"/>
+      <c r="J31" s="30" t="str">
         <f aca="false">IF($I$33=0,"",I31/$I$33)</f>
         <v/>
       </c>
-      <c r="K31" s="28"/>
-      <c r="L31" s="29" t="str">
+      <c r="K31" s="29"/>
+      <c r="L31" s="30" t="str">
         <f aca="false">IF($K$33=0,"",K31/$K$33)</f>
         <v/>
       </c>
-      <c r="M31" s="30" t="n">
+      <c r="M31" s="31" t="n">
         <f aca="false">G31+I31+K31</f>
         <v>0</v>
       </c>
-      <c r="N31" s="29" t="str">
+      <c r="N31" s="30" t="str">
         <f aca="false">IF($M$33=0,"",M31/$M$33)</f>
         <v/>
       </c>
-      <c r="O31" s="28"/>
-      <c r="P31" s="29" t="str">
+      <c r="O31" s="29"/>
+      <c r="P31" s="30" t="str">
         <f aca="false">IF($O$33=0,"",O31/$O$33)</f>
         <v/>
       </c>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="29" t="str">
+      <c r="Q31" s="29"/>
+      <c r="R31" s="30" t="str">
         <f aca="false">IF($Q$33=0,"",Q31/$Q$33)</f>
         <v/>
       </c>
-      <c r="S31" s="28"/>
-      <c r="T31" s="29" t="str">
+      <c r="S31" s="29"/>
+      <c r="T31" s="30" t="str">
         <f aca="false">IF($S$33=0,"",S31/$S$33)</f>
         <v/>
       </c>
-      <c r="U31" s="30" t="n">
+      <c r="U31" s="31" t="n">
         <f aca="false">O31+Q31+S31</f>
         <v>0</v>
       </c>
-      <c r="V31" s="29" t="str">
+      <c r="V31" s="30" t="str">
         <f aca="false">IF($U$33=0,"",U31/$U$33)</f>
         <v/>
       </c>
@@ -4228,122 +4271,122 @@
         <v>18</v>
       </c>
       <c r="B32" s="12"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="29" t="str">
+      <c r="C32" s="29"/>
+      <c r="D32" s="30" t="str">
         <f aca="false">IF($C$33=0,"",C32/$C$33)</f>
         <v/>
       </c>
-      <c r="E32" s="28"/>
-      <c r="F32" s="29" t="str">
+      <c r="E32" s="29"/>
+      <c r="F32" s="30" t="str">
         <f aca="false">IF($E$33=0,"",E32/$E$33)</f>
         <v/>
       </c>
-      <c r="G32" s="28"/>
-      <c r="H32" s="29" t="str">
+      <c r="G32" s="29"/>
+      <c r="H32" s="30" t="str">
         <f aca="false">IF($G$33=0,"",G32/$G$33)</f>
         <v/>
       </c>
-      <c r="I32" s="28"/>
-      <c r="J32" s="29" t="str">
+      <c r="I32" s="29"/>
+      <c r="J32" s="30" t="str">
         <f aca="false">IF($I$33=0,"",I32/$I$33)</f>
         <v/>
       </c>
-      <c r="K32" s="28"/>
-      <c r="L32" s="29" t="str">
+      <c r="K32" s="29"/>
+      <c r="L32" s="30" t="str">
         <f aca="false">IF($K$33=0,"",K32/$K$33)</f>
         <v/>
       </c>
-      <c r="M32" s="30" t="n">
+      <c r="M32" s="31" t="n">
         <f aca="false">G32+I32+K32</f>
         <v>0</v>
       </c>
-      <c r="N32" s="29" t="str">
+      <c r="N32" s="30" t="str">
         <f aca="false">IF($M$33=0,"",M32/$M$33)</f>
         <v/>
       </c>
-      <c r="O32" s="28"/>
-      <c r="P32" s="29" t="str">
+      <c r="O32" s="29"/>
+      <c r="P32" s="30" t="str">
         <f aca="false">IF($O$33=0,"",O32/$O$33)</f>
         <v/>
       </c>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="29" t="str">
+      <c r="Q32" s="29"/>
+      <c r="R32" s="30" t="str">
         <f aca="false">IF($Q$33=0,"",Q32/$Q$33)</f>
         <v/>
       </c>
-      <c r="S32" s="28"/>
-      <c r="T32" s="29" t="str">
+      <c r="S32" s="29"/>
+      <c r="T32" s="30" t="str">
         <f aca="false">IF($S$33=0,"",S32/$S$33)</f>
         <v/>
       </c>
-      <c r="U32" s="30" t="n">
+      <c r="U32" s="31" t="n">
         <f aca="false">O32+Q32+S32</f>
         <v>0</v>
       </c>
-      <c r="V32" s="29" t="str">
+      <c r="V32" s="30" t="str">
         <f aca="false">IF($U$33=0,"",U32/$U$33)</f>
         <v/>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="31" t="n">
+      <c r="A33" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="B33" s="20"/>
+      <c r="C33" s="32" t="n">
         <f aca="false">SUM(C30:C32)</f>
         <v>0</v>
       </c>
-      <c r="D33" s="18"/>
-      <c r="E33" s="31" t="n">
+      <c r="D33" s="21"/>
+      <c r="E33" s="32" t="n">
         <f aca="false">SUM(E30:E32)</f>
         <v>0</v>
       </c>
-      <c r="F33" s="18"/>
-      <c r="G33" s="31" t="n">
+      <c r="F33" s="21"/>
+      <c r="G33" s="32" t="n">
         <f aca="false">SUM(G30:G32)</f>
         <v>0</v>
       </c>
-      <c r="H33" s="18"/>
-      <c r="I33" s="31" t="n">
+      <c r="H33" s="21"/>
+      <c r="I33" s="32" t="n">
         <f aca="false">SUM(I30:I32)</f>
         <v>0</v>
       </c>
-      <c r="J33" s="18"/>
-      <c r="K33" s="31" t="n">
+      <c r="J33" s="21"/>
+      <c r="K33" s="32" t="n">
         <f aca="false">SUM(K30:K32)</f>
         <v>0</v>
       </c>
-      <c r="L33" s="18"/>
-      <c r="M33" s="31" t="n">
+      <c r="L33" s="21"/>
+      <c r="M33" s="32" t="n">
         <f aca="false">SUM(M30:M32)</f>
         <v>0</v>
       </c>
-      <c r="N33" s="18"/>
-      <c r="O33" s="31" t="n">
+      <c r="N33" s="21"/>
+      <c r="O33" s="32" t="n">
         <f aca="false">SUM(O30:O32)</f>
         <v>0</v>
       </c>
-      <c r="P33" s="18"/>
-      <c r="Q33" s="31" t="n">
+      <c r="P33" s="21"/>
+      <c r="Q33" s="32" t="n">
         <f aca="false">SUM(Q30:Q32)</f>
         <v>0</v>
       </c>
-      <c r="R33" s="18"/>
-      <c r="S33" s="31" t="n">
+      <c r="R33" s="21"/>
+      <c r="S33" s="32" t="n">
         <f aca="false">SUM(S30:S32)</f>
         <v>0</v>
       </c>
-      <c r="T33" s="18"/>
-      <c r="U33" s="31" t="n">
+      <c r="T33" s="21"/>
+      <c r="U33" s="32" t="n">
         <f aca="false">SUM(U30:U32)</f>
         <v>0</v>
       </c>
-      <c r="V33" s="18"/>
+      <c r="V33" s="21"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -4369,321 +4412,321 @@
     </row>
     <row r="36" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="I36" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="J36" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="K36" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="E36" s="7" t="s">
+      <c r="L36" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="M36" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="F36" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="G36" s="7" t="s">
+      <c r="N36" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="O36" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="H36" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="I36" s="7" t="s">
+      <c r="P36" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q36" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="J36" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="K36" s="7" t="s">
+      <c r="R36" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="S36" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="L36" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="M36" s="7" t="s">
+      <c r="T36" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="U36" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="N36" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="O36" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="P36" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="Q36" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="R36" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="S36" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="T36" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="U36" s="7" t="s">
-        <v>178</v>
-      </c>
       <c r="V36" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B37" s="12"/>
-      <c r="C37" s="28"/>
-      <c r="D37" s="29" t="str">
+      <c r="C37" s="29"/>
+      <c r="D37" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C37/$C$17)</f>
         <v/>
       </c>
-      <c r="E37" s="28"/>
-      <c r="F37" s="29" t="str">
+      <c r="E37" s="29"/>
+      <c r="F37" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E37/$E$17)</f>
         <v/>
       </c>
-      <c r="G37" s="28"/>
-      <c r="H37" s="29" t="str">
+      <c r="G37" s="29"/>
+      <c r="H37" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G37/$G$17)</f>
         <v/>
       </c>
-      <c r="I37" s="28"/>
-      <c r="J37" s="29" t="str">
+      <c r="I37" s="29"/>
+      <c r="J37" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I37/$I$17)</f>
         <v/>
       </c>
-      <c r="K37" s="28"/>
-      <c r="L37" s="29" t="str">
+      <c r="K37" s="29"/>
+      <c r="L37" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K37/$K$17)</f>
         <v/>
       </c>
-      <c r="M37" s="30" t="n">
+      <c r="M37" s="31" t="n">
         <f aca="false">G37+I37+K37</f>
         <v>0</v>
       </c>
-      <c r="N37" s="29" t="str">
+      <c r="N37" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M37/$M$17)</f>
         <v/>
       </c>
-      <c r="O37" s="28"/>
-      <c r="P37" s="29" t="str">
+      <c r="O37" s="29"/>
+      <c r="P37" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O37/$O$17)</f>
         <v/>
       </c>
-      <c r="Q37" s="28"/>
-      <c r="R37" s="29" t="str">
+      <c r="Q37" s="29"/>
+      <c r="R37" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q37/$Q$17)</f>
         <v/>
       </c>
-      <c r="S37" s="28"/>
-      <c r="T37" s="29" t="str">
+      <c r="S37" s="29"/>
+      <c r="T37" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S37/$S$17)</f>
         <v/>
       </c>
-      <c r="U37" s="30" t="n">
+      <c r="U37" s="31" t="n">
         <f aca="false">O37+Q37+S37</f>
         <v>0</v>
       </c>
-      <c r="V37" s="29" t="str">
+      <c r="V37" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U37/$U$17)</f>
         <v/>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B38" s="12"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="29" t="str">
+      <c r="C38" s="29"/>
+      <c r="D38" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C38/$C$17)</f>
         <v/>
       </c>
-      <c r="E38" s="28"/>
-      <c r="F38" s="29" t="str">
+      <c r="E38" s="29"/>
+      <c r="F38" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E38/$E$17)</f>
         <v/>
       </c>
-      <c r="G38" s="28"/>
-      <c r="H38" s="29" t="str">
+      <c r="G38" s="29"/>
+      <c r="H38" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G38/$G$17)</f>
         <v/>
       </c>
-      <c r="I38" s="28"/>
-      <c r="J38" s="29" t="str">
+      <c r="I38" s="29"/>
+      <c r="J38" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I38/$I$17)</f>
         <v/>
       </c>
-      <c r="K38" s="28"/>
-      <c r="L38" s="29" t="str">
+      <c r="K38" s="29"/>
+      <c r="L38" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K38/$K$17)</f>
         <v/>
       </c>
-      <c r="M38" s="30" t="n">
+      <c r="M38" s="31" t="n">
         <f aca="false">G38+I38+K38</f>
         <v>0</v>
       </c>
-      <c r="N38" s="29" t="str">
+      <c r="N38" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M38/$M$17)</f>
         <v/>
       </c>
-      <c r="O38" s="28"/>
-      <c r="P38" s="29" t="str">
+      <c r="O38" s="29"/>
+      <c r="P38" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O38/$O$17)</f>
         <v/>
       </c>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="29" t="str">
+      <c r="Q38" s="29"/>
+      <c r="R38" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q38/$Q$17)</f>
         <v/>
       </c>
-      <c r="S38" s="28"/>
-      <c r="T38" s="29" t="str">
+      <c r="S38" s="29"/>
+      <c r="T38" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S38/$S$17)</f>
         <v/>
       </c>
-      <c r="U38" s="30" t="n">
+      <c r="U38" s="31" t="n">
         <f aca="false">O38+Q38+S38</f>
         <v>0</v>
       </c>
-      <c r="V38" s="29" t="str">
+      <c r="V38" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U38/$U$17)</f>
         <v/>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B39" s="12"/>
-      <c r="C39" s="28"/>
-      <c r="D39" s="29" t="str">
+      <c r="C39" s="29"/>
+      <c r="D39" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C39/$C$17)</f>
         <v/>
       </c>
-      <c r="E39" s="28"/>
-      <c r="F39" s="29" t="str">
+      <c r="E39" s="29"/>
+      <c r="F39" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E39/$E$17)</f>
         <v/>
       </c>
-      <c r="G39" s="28"/>
-      <c r="H39" s="29" t="str">
+      <c r="G39" s="29"/>
+      <c r="H39" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G39/$G$17)</f>
         <v/>
       </c>
-      <c r="I39" s="28"/>
-      <c r="J39" s="29" t="str">
+      <c r="I39" s="29"/>
+      <c r="J39" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I39/$I$17)</f>
         <v/>
       </c>
-      <c r="K39" s="28"/>
-      <c r="L39" s="29" t="str">
+      <c r="K39" s="29"/>
+      <c r="L39" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K39/$K$17)</f>
         <v/>
       </c>
-      <c r="M39" s="30" t="n">
+      <c r="M39" s="31" t="n">
         <f aca="false">G39+I39+K39</f>
         <v>0</v>
       </c>
-      <c r="N39" s="29" t="str">
+      <c r="N39" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M39/$M$17)</f>
         <v/>
       </c>
-      <c r="O39" s="28"/>
-      <c r="P39" s="29" t="str">
+      <c r="O39" s="29"/>
+      <c r="P39" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O39/$O$17)</f>
         <v/>
       </c>
-      <c r="Q39" s="28"/>
-      <c r="R39" s="29" t="str">
+      <c r="Q39" s="29"/>
+      <c r="R39" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q39/$Q$17)</f>
         <v/>
       </c>
-      <c r="S39" s="28"/>
-      <c r="T39" s="29" t="str">
+      <c r="S39" s="29"/>
+      <c r="T39" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S39/$S$17)</f>
         <v/>
       </c>
-      <c r="U39" s="30" t="n">
+      <c r="U39" s="31" t="n">
         <f aca="false">O39+Q39+S39</f>
         <v>0</v>
       </c>
-      <c r="V39" s="29" t="str">
+      <c r="V39" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U39/$U$17)</f>
         <v/>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B40" s="12"/>
-      <c r="C40" s="28"/>
-      <c r="D40" s="29" t="str">
+      <c r="C40" s="29"/>
+      <c r="D40" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C40/$C$17)</f>
         <v/>
       </c>
-      <c r="E40" s="28"/>
-      <c r="F40" s="29" t="str">
+      <c r="E40" s="29"/>
+      <c r="F40" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E40/$E$17)</f>
         <v/>
       </c>
-      <c r="G40" s="28"/>
-      <c r="H40" s="29" t="str">
+      <c r="G40" s="29"/>
+      <c r="H40" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G40/$G$17)</f>
         <v/>
       </c>
-      <c r="I40" s="28"/>
-      <c r="J40" s="29" t="str">
+      <c r="I40" s="29"/>
+      <c r="J40" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I40/$I$17)</f>
         <v/>
       </c>
-      <c r="K40" s="28"/>
-      <c r="L40" s="29" t="str">
+      <c r="K40" s="29"/>
+      <c r="L40" s="30" t="str">
         <f aca="false">IF($K$17=0,"",K40/$K$17)</f>
         <v/>
       </c>
-      <c r="M40" s="30" t="n">
+      <c r="M40" s="31" t="n">
         <f aca="false">G40+I40+K40</f>
         <v>0</v>
       </c>
-      <c r="N40" s="29" t="str">
+      <c r="N40" s="30" t="str">
         <f aca="false">IF($M$17=0,"",M40/$M$17)</f>
         <v/>
       </c>
-      <c r="O40" s="28"/>
-      <c r="P40" s="29" t="str">
+      <c r="O40" s="29"/>
+      <c r="P40" s="30" t="str">
         <f aca="false">IF($O$17=0,"",O40/$O$17)</f>
         <v/>
       </c>
-      <c r="Q40" s="28"/>
-      <c r="R40" s="29" t="str">
+      <c r="Q40" s="29"/>
+      <c r="R40" s="30" t="str">
         <f aca="false">IF($Q$17=0,"",Q40/$Q$17)</f>
         <v/>
       </c>
-      <c r="S40" s="28"/>
-      <c r="T40" s="29" t="str">
+      <c r="S40" s="29"/>
+      <c r="T40" s="30" t="str">
         <f aca="false">IF($S$17=0,"",S40/$S$17)</f>
         <v/>
       </c>
-      <c r="U40" s="30" t="n">
+      <c r="U40" s="31" t="n">
         <f aca="false">O40+Q40+S40</f>
         <v>0</v>
       </c>
-      <c r="V40" s="29" t="str">
+      <c r="V40" s="30" t="str">
         <f aca="false">IF($U$17=0,"",U40/$U$17)</f>
         <v/>
       </c>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -4709,7 +4752,7 @@
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -4789,12 +4832,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4808,7 +4851,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -4828,28 +4871,28 @@
         <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4857,23 +4900,23 @@
         <v>25</v>
       </c>
       <c r="B7" s="13"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="29" t="str">
+      <c r="C7" s="29"/>
+      <c r="D7" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C7/$C$17)</f>
         <v/>
       </c>
-      <c r="E7" s="28"/>
-      <c r="F7" s="29" t="str">
+      <c r="E7" s="29"/>
+      <c r="F7" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E7/$E$17)</f>
         <v/>
       </c>
-      <c r="G7" s="28"/>
-      <c r="H7" s="29" t="str">
+      <c r="G7" s="29"/>
+      <c r="H7" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G7/$G$17)</f>
         <v/>
       </c>
-      <c r="I7" s="28"/>
-      <c r="J7" s="29" t="str">
+      <c r="I7" s="29"/>
+      <c r="J7" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I7/$I$17)</f>
         <v/>
       </c>
@@ -4885,23 +4928,23 @@
       <c r="B8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="29" t="str">
+      <c r="C8" s="29"/>
+      <c r="D8" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C8/$C$17)</f>
         <v/>
       </c>
-      <c r="E8" s="28"/>
-      <c r="F8" s="29" t="str">
+      <c r="E8" s="29"/>
+      <c r="F8" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E8/$E$17)</f>
         <v/>
       </c>
-      <c r="G8" s="28"/>
-      <c r="H8" s="29" t="str">
+      <c r="G8" s="29"/>
+      <c r="H8" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G8/$G$17)</f>
         <v/>
       </c>
-      <c r="I8" s="28"/>
-      <c r="J8" s="29" t="str">
+      <c r="I8" s="29"/>
+      <c r="J8" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I8/$I$17)</f>
         <v/>
       </c>
@@ -4913,23 +4956,23 @@
       <c r="B9" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="29" t="str">
+      <c r="C9" s="29"/>
+      <c r="D9" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C9/$C$17)</f>
         <v/>
       </c>
-      <c r="E9" s="28"/>
-      <c r="F9" s="29" t="str">
+      <c r="E9" s="29"/>
+      <c r="F9" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E9/$E$17)</f>
         <v/>
       </c>
-      <c r="G9" s="28"/>
-      <c r="H9" s="29" t="str">
+      <c r="G9" s="29"/>
+      <c r="H9" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G9/$G$17)</f>
         <v/>
       </c>
-      <c r="I9" s="28"/>
-      <c r="J9" s="29" t="str">
+      <c r="I9" s="29"/>
+      <c r="J9" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I9/$I$17)</f>
         <v/>
       </c>
@@ -4941,23 +4984,23 @@
       <c r="B10" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="29" t="str">
+      <c r="C10" s="29"/>
+      <c r="D10" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C10/$C$17)</f>
         <v/>
       </c>
-      <c r="E10" s="28"/>
-      <c r="F10" s="29" t="str">
+      <c r="E10" s="29"/>
+      <c r="F10" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E10/$E$17)</f>
         <v/>
       </c>
-      <c r="G10" s="28"/>
-      <c r="H10" s="29" t="str">
+      <c r="G10" s="29"/>
+      <c r="H10" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G10/$G$17)</f>
         <v/>
       </c>
-      <c r="I10" s="28"/>
-      <c r="J10" s="29" t="str">
+      <c r="I10" s="29"/>
+      <c r="J10" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I10/$I$17)</f>
         <v/>
       </c>
@@ -4969,23 +5012,23 @@
       <c r="B11" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="28"/>
-      <c r="D11" s="29" t="str">
+      <c r="C11" s="29"/>
+      <c r="D11" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C11/$C$17)</f>
         <v/>
       </c>
-      <c r="E11" s="28"/>
-      <c r="F11" s="29" t="str">
+      <c r="E11" s="29"/>
+      <c r="F11" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E11/$E$17)</f>
         <v/>
       </c>
-      <c r="G11" s="28"/>
-      <c r="H11" s="29" t="str">
+      <c r="G11" s="29"/>
+      <c r="H11" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G11/$G$17)</f>
         <v/>
       </c>
-      <c r="I11" s="28"/>
-      <c r="J11" s="29" t="str">
+      <c r="I11" s="29"/>
+      <c r="J11" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I11/$I$17)</f>
         <v/>
       </c>
@@ -4997,23 +5040,23 @@
       <c r="B12" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="29" t="str">
+      <c r="C12" s="29"/>
+      <c r="D12" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C12/$C$17)</f>
         <v/>
       </c>
-      <c r="E12" s="28"/>
-      <c r="F12" s="29" t="str">
+      <c r="E12" s="29"/>
+      <c r="F12" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E12/$E$17)</f>
         <v/>
       </c>
-      <c r="G12" s="28"/>
-      <c r="H12" s="29" t="str">
+      <c r="G12" s="29"/>
+      <c r="H12" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G12/$G$17)</f>
         <v/>
       </c>
-      <c r="I12" s="28"/>
-      <c r="J12" s="29" t="str">
+      <c r="I12" s="29"/>
+      <c r="J12" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I12/$I$17)</f>
         <v/>
       </c>
@@ -5025,23 +5068,23 @@
       <c r="B13" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="28"/>
-      <c r="D13" s="29" t="str">
+      <c r="C13" s="29"/>
+      <c r="D13" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C13/$C$17)</f>
         <v/>
       </c>
-      <c r="E13" s="28"/>
-      <c r="F13" s="29" t="str">
+      <c r="E13" s="29"/>
+      <c r="F13" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E13/$E$17)</f>
         <v/>
       </c>
-      <c r="G13" s="28"/>
-      <c r="H13" s="29" t="str">
+      <c r="G13" s="29"/>
+      <c r="H13" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G13/$G$17)</f>
         <v/>
       </c>
-      <c r="I13" s="28"/>
-      <c r="J13" s="29" t="str">
+      <c r="I13" s="29"/>
+      <c r="J13" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I13/$I$17)</f>
         <v/>
       </c>
@@ -5053,23 +5096,23 @@
       <c r="B14" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="29" t="str">
+      <c r="C14" s="29"/>
+      <c r="D14" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C14/$C$17)</f>
         <v/>
       </c>
-      <c r="E14" s="28"/>
-      <c r="F14" s="29" t="str">
+      <c r="E14" s="29"/>
+      <c r="F14" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E14/$E$17)</f>
         <v/>
       </c>
-      <c r="G14" s="28"/>
-      <c r="H14" s="29" t="str">
+      <c r="G14" s="29"/>
+      <c r="H14" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G14/$G$17)</f>
         <v/>
       </c>
-      <c r="I14" s="28"/>
-      <c r="J14" s="29" t="str">
+      <c r="I14" s="29"/>
+      <c r="J14" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I14/$I$17)</f>
         <v/>
       </c>
@@ -5081,23 +5124,23 @@
       <c r="B15" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="29" t="str">
+      <c r="C15" s="29"/>
+      <c r="D15" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C15/$C$17)</f>
         <v/>
       </c>
-      <c r="E15" s="28"/>
-      <c r="F15" s="29" t="str">
+      <c r="E15" s="29"/>
+      <c r="F15" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E15/$E$17)</f>
         <v/>
       </c>
-      <c r="G15" s="28"/>
-      <c r="H15" s="29" t="str">
+      <c r="G15" s="29"/>
+      <c r="H15" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G15/$G$17)</f>
         <v/>
       </c>
-      <c r="I15" s="28"/>
-      <c r="J15" s="29" t="str">
+      <c r="I15" s="29"/>
+      <c r="J15" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I15/$I$17)</f>
         <v/>
       </c>
@@ -5109,52 +5152,52 @@
       <c r="B16" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="28"/>
-      <c r="D16" s="29" t="str">
+      <c r="C16" s="29"/>
+      <c r="D16" s="30" t="str">
         <f aca="false">IF($C$17=0,"",C16/$C$17)</f>
         <v/>
       </c>
-      <c r="E16" s="28"/>
-      <c r="F16" s="29" t="str">
+      <c r="E16" s="29"/>
+      <c r="F16" s="30" t="str">
         <f aca="false">IF($E$17=0,"",E16/$E$17)</f>
         <v/>
       </c>
-      <c r="G16" s="28"/>
-      <c r="H16" s="29" t="str">
+      <c r="G16" s="29"/>
+      <c r="H16" s="30" t="str">
         <f aca="false">IF($G$17=0,"",G16/$G$17)</f>
         <v/>
       </c>
-      <c r="I16" s="28"/>
-      <c r="J16" s="29" t="str">
+      <c r="I16" s="29"/>
+      <c r="J16" s="30" t="str">
         <f aca="false">IF($I$17=0,"",I16/$I$17)</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="31" t="n">
+      <c r="A17" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="B17" s="20"/>
+      <c r="C17" s="32" t="n">
         <f aca="false">SUM(C7:C16)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="18"/>
-      <c r="E17" s="31" t="n">
+      <c r="D17" s="21"/>
+      <c r="E17" s="32" t="n">
         <f aca="false">SUM(E7:E16)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="18"/>
-      <c r="G17" s="31" t="n">
+      <c r="F17" s="21"/>
+      <c r="G17" s="32" t="n">
         <f aca="false">SUM(G7:G16)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="18"/>
-      <c r="I17" s="31" t="n">
+      <c r="H17" s="21"/>
+      <c r="I17" s="32" t="n">
         <f aca="false">SUM(I7:I16)</f>
         <v>0</v>
       </c>
-      <c r="J17" s="18"/>
+      <c r="J17" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
A2: model workbook — reachability rules say confirmed contact (inbound call, successful call or right-party result), not any contact
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -911,7 +911,7 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>The last 3 days we called all failed, with no contact since.</t>
+          <t>The last 3 days we called all failed, with no confirmed contact since.</t>
         </is>
       </c>
       <c r="D15" s="8" t="n"/>
@@ -1268,7 +1268,7 @@
       <c r="B12" s="8" t="n"/>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Confirmed contact</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -1423,12 +1423,12 @@
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>Last contact</t>
+          <t>Last confirmed contact</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Date of the most recent contact.</t>
+          <t>Date of the most recent confirmed contact with the customer.</t>
         </is>
       </c>
       <c r="C23" s="8" t="n"/>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>Last 3 call days all failed, the oldest within the window, and no contact since.</t>
+          <t>Last 3 call days all failed, the oldest within the window, and no confirmed contact since.</t>
         </is>
       </c>
       <c r="C34" s="8" t="n"/>
@@ -1584,7 +1584,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="22" customHeight="1">
+    <row r="35" ht="33" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
           <t>Rule 2</t>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B35" s="21" t="inlineStr">
         <is>
-          <t>Last contact is within the window.</t>
+          <t>The last confirmed contact with the customer (they called us, a call marked successful, or a result only the customer can give) is within the window.</t>
         </is>
       </c>
       <c r="C35" s="8" t="n"/>
@@ -1769,7 +1769,7 @@
     <row r="48" ht="33" customHeight="1">
       <c r="A48" s="22" t="inlineStr">
         <is>
-          <t>Contacts for Reachable</t>
+          <t>Confirmed contacts for Reachable</t>
         </is>
       </c>
       <c r="B48" s="23" t="inlineStr">
@@ -1780,7 +1780,7 @@
       <c r="C48" s="8" t="n"/>
       <c r="D48" s="24" t="inlineStr">
         <is>
-          <t>One recent contact shows they can be reached.</t>
+          <t>One recent confirmed contact shows they can be reached.</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Reachability: no recent contact</t>
+          <t>Reachability: no recent confirmed contact</t>
         </is>
       </c>
       <c r="B40" s="8" t="n"/>

</xml_diff>

<commit_message>
A2: Non-Reachable streak per segment — 6 failed call days at 180+, 3 at 60–180 (GRR, D-A2-20); spec test 36 cases
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -911,7 +911,7 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>The last 3 days we called all failed, with no confirmed contact since.</t>
+          <t>The last 3 days we called (6 at 180+) all failed, with no confirmed contact since.</t>
         </is>
       </c>
       <c r="D15" s="8" t="n"/>
@@ -1441,12 +1441,12 @@
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>Last 3 call days</t>
+          <t>Last call days</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>The 3 most recent days we called, each failed or not.</t>
+          <t>The 3 most recent days we called (6 at 180+), each failed or not.</t>
         </is>
       </c>
       <c r="C24" s="8" t="n"/>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>Last 3 call days all failed, the oldest within the window, and no confirmed contact since.</t>
+          <t>Last 3 call days (6 at 180+) all failed, the oldest within the window, and no confirmed contact since.</t>
         </is>
       </c>
       <c r="C34" s="8" t="n"/>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="60" customHeight="1">
+    <row r="47" ht="73.5" customHeight="1">
       <c r="A47" s="22" t="inlineStr">
         <is>
           <t>Failed call days</t>
@@ -1756,13 +1756,13 @@
       </c>
       <c r="B47" s="23" t="inlineStr">
         <is>
-          <t>The last 3 call days.</t>
+          <t>The last 3 call days at 61–180 DPD, the last 6 at 180+ DPD.</t>
         </is>
       </c>
       <c r="C47" s="8" t="n"/>
       <c r="D47" s="24" t="inlineStr">
         <is>
-          <t>Fewer is not a pattern. 86% of accounts have 6+ call days in 3 months; sensitivity 1–10 days under check.</t>
+          <t>Fewer is not a pattern; 6 at 180+ set by GRR. 86% of accounts at 61–180 have 6+ call days in 3 months; sensitivity 1–10 days under check.</t>
         </is>
       </c>
     </row>
@@ -2996,7 +2996,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="33" customHeight="1">
+    <row r="14" ht="46.5" customHeight="1">
       <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Reachable</t>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>A contact within the window; 3 failed call days after it still make Non-Reachable.</t>
+          <t>A contact within the window; 3 failed call days after it (6 at 180+) still make Non-Reachable.</t>
         </is>
       </c>
       <c r="D14" s="24" t="inlineStr">

</xml_diff>

<commit_message>
A2: bundle 10 rebuilt — Sonnet prompt for the workplace workbook; builder gets the 180+ change row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/locatability/a2_locatability_reference.xlsx
+++ b/docs/locatability/a2_locatability_reference.xlsx
@@ -2753,7 +2753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3043,71 +3043,93 @@
     <row r="16" ht="33" customHeight="1">
       <c r="A16" s="22" t="inlineStr">
         <is>
+          <t>Failed call days at 180+</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>3 call days.</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>6 call days (GRR); 3 at 61–180.</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>None at 61–180; 180+ not run yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="33" customHeight="1">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
           <t>Call history</t>
         </is>
       </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>From the spell start.</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C17" s="23" t="inlineStr">
         <is>
           <t>All collections history up to the scoring date.</t>
         </is>
       </c>
-      <c r="D16" s="24" t="inlineStr">
+      <c r="D17" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="46.5" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+    <row r="18" ht="46.5" customHeight="1">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>Deceased</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B18" s="23" t="inlineStr">
         <is>
           <t>Collector note; card block joined on the exact date.</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C18" s="23" t="inlineStr">
         <is>
           <t>Collector note (claims included), card block D on the latest snapshot, customer record flag.</t>
         </is>
       </c>
-      <c r="D17" s="24" t="inlineStr">
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>44 → 89; 33 of them have no collector note.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="33" customHeight="1">
-      <c r="A18" s="22" t="inlineStr">
+    <row r="19" ht="33" customHeight="1">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
       </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>Routing flags (promise to pay, hardship, refusing, field visit), contact rates.</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
+      <c r="C19" s="23" t="inlineStr">
         <is>
           <t>Left to the other axes.</t>
         </is>
       </c>
-      <c r="D18" s="24" t="inlineStr">
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="19.5" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21" ht="19.5" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Loans: the old output had 111 extra rows from departure spells; the new one covers exactly the scored accounts (3,985).</t>
         </is>
@@ -3115,7 +3137,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>